<commit_message>
logs: update NSE signals 2026-05-25
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Scans" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Signals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Scans" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signals'!$A$1:$V$1</definedName>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -109,6 +109,12 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -179,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -237,6 +243,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -628,6 +637,8 @@
     <col width="11" customWidth="1" min="20" max="20"/>
     <col width="9" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -739,6 +750,16 @@
       <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="W1" s="20" t="inlineStr">
+        <is>
+          <t>India VIX</t>
+        </is>
+      </c>
+      <c r="X1" s="20" t="inlineStr">
+        <is>
+          <t>Nifty PCR</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5820,6 +5841,2080 @@
       <c r="H105" s="11" t="inlineStr">
         <is>
           <t>APOLLOHOSP, ASTRAL, OBEROIRLTY, JUBLFOOD, BOSCHLTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B106" s="12" t="inlineStr">
+        <is>
+          <t>10:22:06</t>
+        </is>
+      </c>
+      <c r="C106" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E106" s="12" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F106" s="12" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G106" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>10:27:07</t>
+        </is>
+      </c>
+      <c r="C107" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D107" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="E107" s="11" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="F107" s="11" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G107" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B108" s="12" t="inlineStr">
+        <is>
+          <t>10:32:08</t>
+        </is>
+      </c>
+      <c r="C108" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D108" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="E108" s="12" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G108" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>10:37:10</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="E109" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F109" s="11" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G109" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B110" s="12" t="inlineStr">
+        <is>
+          <t>10:42:11</t>
+        </is>
+      </c>
+      <c r="C110" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D110" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E110" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="F110" s="12" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G110" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>10:47:12</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D111" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E111" s="11" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G111" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t>10:52:14</t>
+        </is>
+      </c>
+      <c r="C112" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D112" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E112" s="12" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G112" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>10:57:15</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D113" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E113" s="11" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F113" s="11" t="inlineStr">
+        <is>
+          <t>Morning Momentum</t>
+        </is>
+      </c>
+      <c r="G113" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B114" s="12" t="inlineStr">
+        <is>
+          <t>11:02:16</t>
+        </is>
+      </c>
+      <c r="C114" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D114" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="E114" s="12" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G114" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>11:07:18</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D115" s="11" t="n">
+        <v>73</v>
+      </c>
+      <c r="E115" s="11" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="F115" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G115" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t>11:12:19</t>
+        </is>
+      </c>
+      <c r="C116" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D116" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E116" s="12" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G116" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>11:17:20</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D117" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="E117" s="11" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G117" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>11:22:22</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D118" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="E118" s="12" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G118" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>11:27:23</t>
+        </is>
+      </c>
+      <c r="C119" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D119" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="E119" s="11" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G119" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>11:32:24</t>
+        </is>
+      </c>
+      <c r="C120" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D120" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="E120" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G120" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>11:37:26</t>
+        </is>
+      </c>
+      <c r="C121" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D121" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E121" s="11" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="F121" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G121" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B122" s="12" t="inlineStr">
+        <is>
+          <t>11:42:27</t>
+        </is>
+      </c>
+      <c r="C122" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D122" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="E122" s="12" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G122" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>11:47:28</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D123" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E123" s="11" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F123" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B124" s="12" t="inlineStr">
+        <is>
+          <t>11:52:30</t>
+        </is>
+      </c>
+      <c r="C124" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D124" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="E124" s="12" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G124" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>11:57:31</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D125" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="E125" s="11" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G125" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>12:02:31</t>
+        </is>
+      </c>
+      <c r="C126" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D126" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="E126" s="12" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G126" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>12:07:33</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D127" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E127" s="11" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="F127" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G127" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t>12:12:34</t>
+        </is>
+      </c>
+      <c r="C128" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D128" s="12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E128" s="12" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>12:17:35</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D129" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="E129" s="11" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F129" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G129" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t>12:22:37</t>
+        </is>
+      </c>
+      <c r="C130" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D130" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="E130" s="12" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G130" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>12:27:38</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D131" s="11" t="n">
+        <v>67</v>
+      </c>
+      <c r="E131" s="11" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F131" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G131" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>12:32:39</t>
+        </is>
+      </c>
+      <c r="C132" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="D132" s="12" t="n">
+        <v>67</v>
+      </c>
+      <c r="E132" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G132" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>12:37:41</t>
+        </is>
+      </c>
+      <c r="C133" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D133" s="11" t="n">
+        <v>69</v>
+      </c>
+      <c r="E133" s="11" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F133" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G133" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t>12:42:42</t>
+        </is>
+      </c>
+      <c r="C134" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D134" s="12" t="n">
+        <v>71</v>
+      </c>
+      <c r="E134" s="12" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G134" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>12:47:43</t>
+        </is>
+      </c>
+      <c r="C135" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D135" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E135" s="11" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="F135" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G135" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B136" s="12" t="inlineStr">
+        <is>
+          <t>12:52:46</t>
+        </is>
+      </c>
+      <c r="C136" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D136" s="12" t="n">
+        <v>69</v>
+      </c>
+      <c r="E136" s="12" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G136" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>12:57:47</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D137" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E137" s="11" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G137" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t>13:02:48</t>
+        </is>
+      </c>
+      <c r="C138" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D138" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E138" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G138" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>13:07:51</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="D139" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="E139" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G139" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>13:12:52</t>
+        </is>
+      </c>
+      <c r="C140" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="D140" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="E140" s="12" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G140" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>13:17:53</t>
+        </is>
+      </c>
+      <c r="C141" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="D141" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="E141" s="11" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="F141" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G141" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>13:22:54</t>
+        </is>
+      </c>
+      <c r="C142" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="D142" s="12" t="n">
+        <v>77</v>
+      </c>
+      <c r="E142" s="12" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>13:27:56</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="n">
+        <v>38</v>
+      </c>
+      <c r="D143" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="E143" s="11" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G143" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="C144" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="D144" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E144" s="12" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G144" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B145" s="11" t="inlineStr">
+        <is>
+          <t>13:38:00</t>
+        </is>
+      </c>
+      <c r="C145" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="D145" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E145" s="11" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="F145" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G145" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>13:43:01</t>
+        </is>
+      </c>
+      <c r="C146" s="12" t="n">
+        <v>41</v>
+      </c>
+      <c r="D146" s="12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E146" s="12" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G146" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>13:48:02</t>
+        </is>
+      </c>
+      <c r="C147" s="11" t="n">
+        <v>42</v>
+      </c>
+      <c r="D147" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="E147" s="11" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="F147" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G147" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>13:53:04</t>
+        </is>
+      </c>
+      <c r="C148" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="D148" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="E148" s="12" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="F148" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G148" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>13:58:05</t>
+        </is>
+      </c>
+      <c r="C149" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="D149" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E149" s="11" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F149" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G149" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>14:03:06</t>
+        </is>
+      </c>
+      <c r="C150" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="D150" s="12" t="n">
+        <v>72</v>
+      </c>
+      <c r="E150" s="12" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F150" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G150" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B151" s="11" t="inlineStr">
+        <is>
+          <t>14:08:08</t>
+        </is>
+      </c>
+      <c r="C151" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="D151" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="E151" s="11" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F151" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G151" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B152" s="12" t="inlineStr">
+        <is>
+          <t>14:13:09</t>
+        </is>
+      </c>
+      <c r="C152" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="D152" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="E152" s="12" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F152" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G152" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B153" s="11" t="inlineStr">
+        <is>
+          <t>14:18:11</t>
+        </is>
+      </c>
+      <c r="C153" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="D153" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="E153" s="11" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F153" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G153" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B154" s="12" t="inlineStr">
+        <is>
+          <t>14:23:13</t>
+        </is>
+      </c>
+      <c r="C154" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="D154" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="E154" s="12" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F154" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G154" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>14:28:14</t>
+        </is>
+      </c>
+      <c r="C155" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="D155" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="E155" s="11" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F155" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G155" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>14:33:15</t>
+        </is>
+      </c>
+      <c r="C156" s="12" t="n">
+        <v>51</v>
+      </c>
+      <c r="D156" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="E156" s="12" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="F156" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G156" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B157" s="11" t="inlineStr">
+        <is>
+          <t>14:38:17</t>
+        </is>
+      </c>
+      <c r="C157" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="D157" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="E157" s="11" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="F157" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G157" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B158" s="12" t="inlineStr">
+        <is>
+          <t>14:43:18</t>
+        </is>
+      </c>
+      <c r="C158" s="12" t="n">
+        <v>53</v>
+      </c>
+      <c r="D158" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="E158" s="12" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="F158" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G158" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B159" s="11" t="inlineStr">
+        <is>
+          <t>14:48:19</t>
+        </is>
+      </c>
+      <c r="C159" s="11" t="n">
+        <v>54</v>
+      </c>
+      <c r="D159" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="E159" s="11" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="F159" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G159" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t>14:53:21</t>
+        </is>
+      </c>
+      <c r="C160" s="12" t="n">
+        <v>55</v>
+      </c>
+      <c r="D160" s="12" t="n">
+        <v>80</v>
+      </c>
+      <c r="E160" s="12" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F160" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G160" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>14:58:22</t>
+        </is>
+      </c>
+      <c r="C161" s="11" t="n">
+        <v>56</v>
+      </c>
+      <c r="D161" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="E161" s="11" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F161" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G161" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B162" s="12" t="inlineStr">
+        <is>
+          <t>15:03:23</t>
+        </is>
+      </c>
+      <c r="C162" s="12" t="n">
+        <v>57</v>
+      </c>
+      <c r="D162" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="E162" s="12" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F162" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G162" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B163" s="11" t="inlineStr">
+        <is>
+          <t>15:08:25</t>
+        </is>
+      </c>
+      <c r="C163" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="D163" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="E163" s="11" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="F163" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G163" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B164" s="12" t="inlineStr">
+        <is>
+          <t>15:13:26</t>
+        </is>
+      </c>
+      <c r="C164" s="12" t="n">
+        <v>59</v>
+      </c>
+      <c r="D164" s="12" t="n">
+        <v>79</v>
+      </c>
+      <c r="E164" s="12" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F164" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G164" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>15:18:28</t>
+        </is>
+      </c>
+      <c r="C165" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="D165" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="E165" s="11" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="F165" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G165" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="B166" s="12" t="inlineStr">
+        <is>
+          <t>15:23:30</t>
+        </is>
+      </c>
+      <c r="C166" s="12" t="n">
+        <v>61</v>
+      </c>
+      <c r="D166" s="12" t="n">
+        <v>78</v>
+      </c>
+      <c r="E166" s="12" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="F166" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G166" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-08
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,8 +612,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:X22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -709,12 +709,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>SL (Rs)</t>
+          <t>SL Price</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Target (Rs)</t>
+          <t>Target Price</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Trade Outcome</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -2238,10 +2238,18 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-08  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A22:X22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2254,7 +2262,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H166"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -7930,8 +7938,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -8087,6 +8095,36 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-09
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,8 +612,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:X23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -2245,11 +2245,19 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-09  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A22:X22"/>
+    <mergeCell ref="A23:X23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2262,7 +2270,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H166"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -7938,8 +7946,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -8125,6 +8133,36 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-10
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X23"/>
+  <dimension ref="A1:X24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2252,10 +2252,18 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-10  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A24:X24"/>
     <mergeCell ref="A22:X22"/>
     <mergeCell ref="A23:X23"/>
   </mergeCells>
@@ -7946,7 +7954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8163,6 +8171,36 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-11
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X24"/>
+  <dimension ref="A1:X25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2259,13 +2259,21 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-11  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
-    <mergeCell ref="A24:X24"/>
     <mergeCell ref="A22:X22"/>
-    <mergeCell ref="A23:X23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2277,7 +2285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7942,6 +7950,550 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B167" s="11" t="inlineStr">
+        <is>
+          <t>14:12:38</t>
+        </is>
+      </c>
+      <c r="C167" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="11" t="n">
+        <v>187</v>
+      </c>
+      <c r="E167" s="11" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="F167" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G167" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B168" s="12" t="inlineStr">
+        <is>
+          <t>14:17:41</t>
+        </is>
+      </c>
+      <c r="C168" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" s="12" t="n">
+        <v>187</v>
+      </c>
+      <c r="E168" s="12" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="F168" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G168" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B169" s="11" t="inlineStr">
+        <is>
+          <t>14:22:55</t>
+        </is>
+      </c>
+      <c r="C169" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D169" s="11" t="n">
+        <v>188</v>
+      </c>
+      <c r="E169" s="11" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="F169" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G169" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t>14:28:00</t>
+        </is>
+      </c>
+      <c r="C170" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D170" s="12" t="n">
+        <v>189</v>
+      </c>
+      <c r="E170" s="12" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="F170" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G170" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>14:33:05</t>
+        </is>
+      </c>
+      <c r="C171" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D171" s="11" t="n">
+        <v>185</v>
+      </c>
+      <c r="E171" s="11" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="F171" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G171" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B172" s="12" t="inlineStr">
+        <is>
+          <t>14:38:10</t>
+        </is>
+      </c>
+      <c r="C172" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D172" s="12" t="n">
+        <v>186</v>
+      </c>
+      <c r="E172" s="12" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="F172" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G172" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>14:43:15</t>
+        </is>
+      </c>
+      <c r="C173" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D173" s="11" t="n">
+        <v>185</v>
+      </c>
+      <c r="E173" s="11" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="F173" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G173" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B174" s="12" t="inlineStr">
+        <is>
+          <t>14:48:19</t>
+        </is>
+      </c>
+      <c r="C174" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D174" s="12" t="n">
+        <v>187</v>
+      </c>
+      <c r="E174" s="12" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="F174" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G174" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B175" s="11" t="inlineStr">
+        <is>
+          <t>14:53:22</t>
+        </is>
+      </c>
+      <c r="C175" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D175" s="11" t="n">
+        <v>191</v>
+      </c>
+      <c r="E175" s="11" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="F175" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G175" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>14:58:28</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D176" s="12" t="n">
+        <v>189</v>
+      </c>
+      <c r="E176" s="12" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F176" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G176" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B177" s="11" t="inlineStr">
+        <is>
+          <t>15:03:32</t>
+        </is>
+      </c>
+      <c r="C177" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D177" s="11" t="n">
+        <v>185</v>
+      </c>
+      <c r="E177" s="11" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="F177" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G177" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B178" s="12" t="inlineStr">
+        <is>
+          <t>15:08:36</t>
+        </is>
+      </c>
+      <c r="C178" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D178" s="12" t="n">
+        <v>187</v>
+      </c>
+      <c r="E178" s="12" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="F178" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B179" s="11" t="inlineStr">
+        <is>
+          <t>15:13:41</t>
+        </is>
+      </c>
+      <c r="C179" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D179" s="11" t="n">
+        <v>191</v>
+      </c>
+      <c r="E179" s="11" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="F179" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G179" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B180" s="12" t="inlineStr">
+        <is>
+          <t>15:18:44</t>
+        </is>
+      </c>
+      <c r="C180" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D180" s="12" t="n">
+        <v>192</v>
+      </c>
+      <c r="E180" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="F180" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G180" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B181" s="11" t="inlineStr">
+        <is>
+          <t>15:23:50</t>
+        </is>
+      </c>
+      <c r="C181" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D181" s="11" t="n">
+        <v>195</v>
+      </c>
+      <c r="E181" s="11" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="F181" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G181" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B182" s="12" t="inlineStr">
+        <is>
+          <t>15:28:55</t>
+        </is>
+      </c>
+      <c r="C182" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D182" s="12" t="n">
+        <v>195</v>
+      </c>
+      <c r="E182" s="12" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="F182" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G182" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7954,7 +8506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8201,6 +8753,36 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-12
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X25"/>
+  <dimension ref="A1:X26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2266,9 +2266,17 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-12  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A23:X23"/>
@@ -8506,7 +8514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8783,6 +8791,36 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-15
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -612,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X26"/>
+  <dimension ref="A1:X27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2273,9 +2273,17 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-15  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A27:X27"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A25:X25"/>
@@ -8514,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8821,6 +8829,36 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-06-16 09:11 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -10,10 +10,12 @@
     <sheet name="Signals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="All Scans" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pre-Open" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signals'!$A$1:$V$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Scans'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pre-Open'!$A$1:$S$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -185,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -246,6 +248,12 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8862,4 +8870,210 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Expiry</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>IEP Gap %</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>BSR</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Depth Imb</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>ATO Net</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>52W Pos %</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
+        <is>
+          <t>Final Qty</t>
+        </is>
+      </c>
+      <c r="L1" s="20" t="inlineStr">
+        <is>
+          <t>Pre-Open Score</t>
+        </is>
+      </c>
+      <c r="M1" s="20" t="inlineStr">
+        <is>
+          <t>Conviction</t>
+        </is>
+      </c>
+      <c r="N1" s="20" t="inlineStr">
+        <is>
+          <t>OI Confirmed</t>
+        </is>
+      </c>
+      <c r="O1" s="20" t="inlineStr">
+        <is>
+          <t>OI Change %</t>
+        </is>
+      </c>
+      <c r="P1" s="20" t="inlineStr">
+        <is>
+          <t>Vol Change %</t>
+        </is>
+      </c>
+      <c r="Q1" s="20" t="inlineStr">
+        <is>
+          <t>LTP</t>
+        </is>
+      </c>
+      <c r="R1" s="20" t="inlineStr">
+        <is>
+          <t>Buildup</t>
+        </is>
+      </c>
+      <c r="S1" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>PGEL</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F2" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K2" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="22" t="n">
+        <v>31.72</v>
+      </c>
+      <c r="M2" s="22" t="inlineStr"/>
+      <c r="N2" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O2" s="22" t="n">
+        <v>5.43</v>
+      </c>
+      <c r="P2" s="22" t="n">
+        <v>113</v>
+      </c>
+      <c r="Q2" s="22" t="n">
+        <v>528.55</v>
+      </c>
+      <c r="R2" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S2" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-16
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X27"/>
+  <dimension ref="A1:X28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2288,13 +2288,21 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-16  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A28:X28"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A22:X22"/>
@@ -8530,7 +8538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8862,6 +8870,36 @@
         <v>0</v>
       </c>
       <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-17
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X28"/>
+  <dimension ref="A1:X29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2295,10 +2295,18 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-17  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A29:X29"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A25:X25"/>
@@ -8538,7 +8546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8900,6 +8908,36 @@
         <v>0</v>
       </c>
       <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-06-18 08:26 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -8954,7 +8954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9148,6 +9148,225 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C3" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="E3" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="22" t="n">
+        <v>80</v>
+      </c>
+      <c r="M3" s="22" t="inlineStr"/>
+      <c r="N3" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O3" s="22" t="n">
+        <v>71.56999999999999</v>
+      </c>
+      <c r="P3" s="22" t="n">
+        <v>1893.1</v>
+      </c>
+      <c r="Q3" s="22" t="n">
+        <v>3703</v>
+      </c>
+      <c r="R3" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S3" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>NYKAA</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="22" t="n">
+        <v>56.84</v>
+      </c>
+      <c r="M4" s="22" t="inlineStr"/>
+      <c r="N4" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O4" s="22" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="P4" s="22" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q4" s="22" t="n">
+        <v>301.3</v>
+      </c>
+      <c r="R4" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S4" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>RVNL</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="22" t="n">
+        <v>35.84</v>
+      </c>
+      <c r="M5" s="22" t="inlineStr"/>
+      <c r="N5" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O5" s="22" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="Q5" s="22" t="n">
+        <v>246.42</v>
+      </c>
+      <c r="R5" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S5" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-18
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -620,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X29"/>
+  <dimension ref="A1:X30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2302,10 +2302,18 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-18  End of Day  |  Signals: 3  |  Stocks: ADANIENT, ADANIENSOL, COCHINSHIP  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A30:X30"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
@@ -2325,7 +2333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H182"/>
+  <dimension ref="A1:H198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8534,6 +8542,550 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B183" s="11" t="inlineStr">
+        <is>
+          <t>14:12:06</t>
+        </is>
+      </c>
+      <c r="C183" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" s="11" t="n">
+        <v>176</v>
+      </c>
+      <c r="E183" s="11" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="F183" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G183" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B184" s="12" t="inlineStr">
+        <is>
+          <t>14:17:08</t>
+        </is>
+      </c>
+      <c r="C184" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D184" s="12" t="n">
+        <v>176</v>
+      </c>
+      <c r="E184" s="12" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="F184" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G184" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B185" s="11" t="inlineStr">
+        <is>
+          <t>14:22:12</t>
+        </is>
+      </c>
+      <c r="C185" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D185" s="11" t="n">
+        <v>175</v>
+      </c>
+      <c r="E185" s="11" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F185" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G185" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t>14:27:17</t>
+        </is>
+      </c>
+      <c r="C186" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D186" s="12" t="n">
+        <v>174</v>
+      </c>
+      <c r="E186" s="12" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F186" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G186" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H186" s="12" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B187" s="11" t="inlineStr">
+        <is>
+          <t>14:32:22</t>
+        </is>
+      </c>
+      <c r="C187" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D187" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="E187" s="11" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="F187" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G187" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H187" s="11" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B188" s="12" t="inlineStr">
+        <is>
+          <t>14:37:26</t>
+        </is>
+      </c>
+      <c r="C188" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D188" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E188" s="12" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="F188" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G188" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H188" s="12" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B189" s="11" t="inlineStr">
+        <is>
+          <t>14:42:32</t>
+        </is>
+      </c>
+      <c r="C189" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D189" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="E189" s="11" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F189" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G189" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H189" s="11" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B190" s="12" t="inlineStr">
+        <is>
+          <t>14:47:39</t>
+        </is>
+      </c>
+      <c r="C190" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D190" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E190" s="12" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="F190" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G190" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H190" s="12" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B191" s="11" t="inlineStr">
+        <is>
+          <t>14:52:43</t>
+        </is>
+      </c>
+      <c r="C191" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D191" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="E191" s="11" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="F191" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G191" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H191" s="11" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B192" s="12" t="inlineStr">
+        <is>
+          <t>14:57:48</t>
+        </is>
+      </c>
+      <c r="C192" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D192" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E192" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="F192" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G192" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H192" s="12" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B193" s="11" t="inlineStr">
+        <is>
+          <t>15:02:54</t>
+        </is>
+      </c>
+      <c r="C193" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D193" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="E193" s="11" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="F193" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G193" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H193" s="11" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B194" s="12" t="inlineStr">
+        <is>
+          <t>15:07:58</t>
+        </is>
+      </c>
+      <c r="C194" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D194" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="E194" s="12" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F194" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G194" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H194" s="12" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B195" s="11" t="inlineStr">
+        <is>
+          <t>15:13:03</t>
+        </is>
+      </c>
+      <c r="C195" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D195" s="11" t="n">
+        <v>179</v>
+      </c>
+      <c r="E195" s="11" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F195" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G195" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" s="11" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B196" s="12" t="inlineStr">
+        <is>
+          <t>15:18:08</t>
+        </is>
+      </c>
+      <c r="C196" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D196" s="12" t="n">
+        <v>179</v>
+      </c>
+      <c r="E196" s="12" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="F196" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G196" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H196" s="12" t="inlineStr">
+        <is>
+          <t>ADANIENT, ADANIENSOL, COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B197" s="11" t="inlineStr">
+        <is>
+          <t>15:23:12</t>
+        </is>
+      </c>
+      <c r="C197" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D197" s="11" t="n">
+        <v>182</v>
+      </c>
+      <c r="E197" s="11" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="F197" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G197" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H197" s="11" t="inlineStr">
+        <is>
+          <t>ADANIENT, ADANIENSOL, COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B198" s="12" t="inlineStr">
+        <is>
+          <t>15:28:17</t>
+        </is>
+      </c>
+      <c r="C198" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D198" s="12" t="n">
+        <v>182</v>
+      </c>
+      <c r="E198" s="12" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F198" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G198" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H198" s="12" t="inlineStr">
+        <is>
+          <t>ADANIENT, ADANIENSOL, COCHINSHIP</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8546,7 +9098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8938,6 +9490,36 @@
         <v>0</v>
       </c>
       <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-06-19 08:54 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -187,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -253,6 +253,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -9536,7 +9542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9949,6 +9955,225 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="24" t="n">
+        <v>67.08</v>
+      </c>
+      <c r="M6" s="24" t="inlineStr"/>
+      <c r="N6" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O6" s="24" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="P6" s="24" t="n">
+        <v>122.4</v>
+      </c>
+      <c r="Q6" s="24" t="n">
+        <v>4739</v>
+      </c>
+      <c r="R6" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S6" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="24" t="n">
+        <v>60.12</v>
+      </c>
+      <c r="M7" s="24" t="inlineStr"/>
+      <c r="N7" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O7" s="24" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="P7" s="24" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="Q7" s="24" t="n">
+        <v>3106.3</v>
+      </c>
+      <c r="R7" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S7" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K8" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="24" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M8" s="24" t="inlineStr"/>
+      <c r="N8" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O8" s="24" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="P8" s="24" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="Q8" s="24" t="n">
+        <v>1041.6</v>
+      </c>
+      <c r="R8" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S8" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-19
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X30"/>
+  <dimension ref="A1:X31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2315,9 +2315,16 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-19  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A29:X29"/>
@@ -2327,6 +2334,7 @@
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A31:X31"/>
     <mergeCell ref="A22:X22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9104,7 +9112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9526,6 +9534,36 @@
         <v>0</v>
       </c>
       <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-22
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X31"/>
+  <dimension ref="A1:X32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2322,14 +2322,22 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-22  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A32:X32"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A23:X23"/>
@@ -9112,7 +9120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9564,6 +9572,36 @@
         <v>0</v>
       </c>
       <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-23
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X32"/>
+  <dimension ref="A1:X33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2329,9 +2329,16 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-23  End of Day  |  Signals: 4  |  Stocks: POLICYBZR, NMDC, ADANIGREEN, GVT&amp;D  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A29:X29"/>
@@ -2340,6 +2347,7 @@
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A33:X33"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A31:X31"/>
@@ -2355,7 +2363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9108,6 +9116,958 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B199" s="11" t="inlineStr">
+        <is>
+          <t>13:14:06</t>
+        </is>
+      </c>
+      <c r="C199" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" s="11" t="n">
+        <v>142</v>
+      </c>
+      <c r="E199" s="11" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="F199" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G199" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B200" s="12" t="inlineStr">
+        <is>
+          <t>13:19:08</t>
+        </is>
+      </c>
+      <c r="C200" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D200" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="E200" s="12" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F200" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G200" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H200" s="12" t="inlineStr">
+        <is>
+          <t>GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B201" s="11" t="inlineStr">
+        <is>
+          <t>13:24:12</t>
+        </is>
+      </c>
+      <c r="C201" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D201" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="E201" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="F201" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G201" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H201" s="11" t="inlineStr">
+        <is>
+          <t>GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B202" s="12" t="inlineStr">
+        <is>
+          <t>13:29:17</t>
+        </is>
+      </c>
+      <c r="C202" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D202" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="E202" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="F202" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G202" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H202" s="12" t="inlineStr">
+        <is>
+          <t>GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B203" s="11" t="inlineStr">
+        <is>
+          <t>13:34:20</t>
+        </is>
+      </c>
+      <c r="C203" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D203" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="E203" s="11" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="F203" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G203" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H203" s="11" t="inlineStr">
+        <is>
+          <t>GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B204" s="12" t="inlineStr">
+        <is>
+          <t>13:39:24</t>
+        </is>
+      </c>
+      <c r="C204" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D204" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="E204" s="12" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F204" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G204" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H204" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B205" s="11" t="inlineStr">
+        <is>
+          <t>13:44:29</t>
+        </is>
+      </c>
+      <c r="C205" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D205" s="11" t="n">
+        <v>139</v>
+      </c>
+      <c r="E205" s="11" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="F205" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G205" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H205" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B206" s="12" t="inlineStr">
+        <is>
+          <t>13:49:32</t>
+        </is>
+      </c>
+      <c r="C206" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D206" s="12" t="n">
+        <v>139</v>
+      </c>
+      <c r="E206" s="12" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F206" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G206" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H206" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B207" s="11" t="inlineStr">
+        <is>
+          <t>13:54:36</t>
+        </is>
+      </c>
+      <c r="C207" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D207" s="11" t="n">
+        <v>141</v>
+      </c>
+      <c r="E207" s="11" t="n">
+        <v>51</v>
+      </c>
+      <c r="F207" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G207" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H207" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B208" s="12" t="inlineStr">
+        <is>
+          <t>13:59:40</t>
+        </is>
+      </c>
+      <c r="C208" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D208" s="12" t="n">
+        <v>141</v>
+      </c>
+      <c r="E208" s="12" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="F208" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G208" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H208" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B209" s="11" t="inlineStr">
+        <is>
+          <t>14:04:44</t>
+        </is>
+      </c>
+      <c r="C209" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D209" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="E209" s="11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="F209" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G209" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H209" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B210" s="12" t="inlineStr">
+        <is>
+          <t>14:09:47</t>
+        </is>
+      </c>
+      <c r="C210" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D210" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="E210" s="12" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F210" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G210" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H210" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B211" s="11" t="inlineStr">
+        <is>
+          <t>14:14:51</t>
+        </is>
+      </c>
+      <c r="C211" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D211" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="E211" s="11" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="F211" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G211" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H211" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B212" s="12" t="inlineStr">
+        <is>
+          <t>14:19:54</t>
+        </is>
+      </c>
+      <c r="C212" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D212" s="12" t="n">
+        <v>144</v>
+      </c>
+      <c r="E212" s="12" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F212" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G212" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H212" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B213" s="11" t="inlineStr">
+        <is>
+          <t>14:24:58</t>
+        </is>
+      </c>
+      <c r="C213" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D213" s="11" t="n">
+        <v>144</v>
+      </c>
+      <c r="E213" s="11" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F213" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G213" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H213" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B214" s="12" t="inlineStr">
+        <is>
+          <t>14:30:02</t>
+        </is>
+      </c>
+      <c r="C214" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D214" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="E214" s="12" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F214" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G214" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H214" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B215" s="11" t="inlineStr">
+        <is>
+          <t>14:35:05</t>
+        </is>
+      </c>
+      <c r="C215" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="D215" s="11" t="n">
+        <v>143</v>
+      </c>
+      <c r="E215" s="11" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="F215" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G215" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H215" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B216" s="12" t="inlineStr">
+        <is>
+          <t>14:40:08</t>
+        </is>
+      </c>
+      <c r="C216" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D216" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="E216" s="12" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="F216" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G216" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H216" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B217" s="11" t="inlineStr">
+        <is>
+          <t>14:45:12</t>
+        </is>
+      </c>
+      <c r="C217" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="D217" s="11" t="n">
+        <v>147</v>
+      </c>
+      <c r="E217" s="11" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="F217" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G217" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H217" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B218" s="12" t="inlineStr">
+        <is>
+          <t>14:50:15</t>
+        </is>
+      </c>
+      <c r="C218" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D218" s="12" t="n">
+        <v>147</v>
+      </c>
+      <c r="E218" s="12" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="F218" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G218" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H218" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B219" s="11" t="inlineStr">
+        <is>
+          <t>14:55:18</t>
+        </is>
+      </c>
+      <c r="C219" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="D219" s="11" t="n">
+        <v>145</v>
+      </c>
+      <c r="E219" s="11" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="F219" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G219" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H219" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B220" s="12" t="inlineStr">
+        <is>
+          <t>15:00:23</t>
+        </is>
+      </c>
+      <c r="C220" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="D220" s="12" t="n">
+        <v>146</v>
+      </c>
+      <c r="E220" s="12" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F220" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G220" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H220" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B221" s="11" t="inlineStr">
+        <is>
+          <t>15:05:26</t>
+        </is>
+      </c>
+      <c r="C221" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="D221" s="11" t="n">
+        <v>145</v>
+      </c>
+      <c r="E221" s="11" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="F221" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G221" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H221" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B222" s="12" t="inlineStr">
+        <is>
+          <t>15:10:29</t>
+        </is>
+      </c>
+      <c r="C222" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="D222" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="E222" s="12" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="F222" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G222" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H222" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B223" s="11" t="inlineStr">
+        <is>
+          <t>15:15:33</t>
+        </is>
+      </c>
+      <c r="C223" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D223" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="E223" s="11" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="F223" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G223" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H223" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B224" s="12" t="inlineStr">
+        <is>
+          <t>15:20:36</t>
+        </is>
+      </c>
+      <c r="C224" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D224" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="E224" s="12" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="F224" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G224" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H224" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B225" s="11" t="inlineStr">
+        <is>
+          <t>15:25:41</t>
+        </is>
+      </c>
+      <c r="C225" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D225" s="11" t="n">
+        <v>149</v>
+      </c>
+      <c r="E225" s="11" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="F225" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G225" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H225" s="11" t="inlineStr">
+        <is>
+          <t>POLICYBZR, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B226" s="12" t="inlineStr">
+        <is>
+          <t>15:30:45</t>
+        </is>
+      </c>
+      <c r="C226" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="D226" s="12" t="n">
+        <v>146</v>
+      </c>
+      <c r="E226" s="12" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="F226" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G226" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H226" s="12" t="inlineStr">
+        <is>
+          <t>POLICYBZR, NMDC, ADANIGREEN, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9120,7 +10080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9602,6 +10562,36 @@
         <v>0</v>
       </c>
       <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-24
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:X34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2336,11 +2336,19 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-24  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
+    <mergeCell ref="A34:X34"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
@@ -10080,7 +10088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10592,6 +10600,36 @@
         <v>0</v>
       </c>
       <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>29</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-25
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X34"/>
+  <dimension ref="A1:X35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2343,13 +2343,21 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-25  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A34:X34"/>
     <mergeCell ref="A29:X29"/>
+    <mergeCell ref="A35:X35"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A32:X32"/>
@@ -2371,7 +2379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H226"/>
+  <dimension ref="A1:H255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10076,6 +10084,992 @@
         </is>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B227" s="11" t="inlineStr">
+        <is>
+          <t>13:09:08</t>
+        </is>
+      </c>
+      <c r="C227" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D227" s="11" t="n">
+        <v>89</v>
+      </c>
+      <c r="E227" s="11" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="F227" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G227" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B228" s="12" t="inlineStr">
+        <is>
+          <t>13:14:10</t>
+        </is>
+      </c>
+      <c r="C228" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D228" s="12" t="n">
+        <v>94</v>
+      </c>
+      <c r="E228" s="12" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="F228" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G228" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H228" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B229" s="11" t="inlineStr">
+        <is>
+          <t>13:19:15</t>
+        </is>
+      </c>
+      <c r="C229" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D229" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="E229" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="F229" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G229" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B230" s="12" t="inlineStr">
+        <is>
+          <t>13:24:19</t>
+        </is>
+      </c>
+      <c r="C230" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D230" s="12" t="n">
+        <v>87</v>
+      </c>
+      <c r="E230" s="12" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F230" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G230" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B231" s="11" t="inlineStr">
+        <is>
+          <t>13:29:22</t>
+        </is>
+      </c>
+      <c r="C231" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D231" s="11" t="n">
+        <v>89</v>
+      </c>
+      <c r="E231" s="11" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="F231" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G231" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B232" s="12" t="inlineStr">
+        <is>
+          <t>13:34:25</t>
+        </is>
+      </c>
+      <c r="C232" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D232" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="E232" s="12" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="F232" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G232" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B233" s="11" t="inlineStr">
+        <is>
+          <t>13:39:29</t>
+        </is>
+      </c>
+      <c r="C233" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D233" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="E233" s="11" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="F233" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G233" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B234" s="12" t="inlineStr">
+        <is>
+          <t>13:44:32</t>
+        </is>
+      </c>
+      <c r="C234" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="D234" s="12" t="n">
+        <v>92</v>
+      </c>
+      <c r="E234" s="12" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="F234" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G234" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B235" s="11" t="inlineStr">
+        <is>
+          <t>13:49:36</t>
+        </is>
+      </c>
+      <c r="C235" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D235" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="E235" s="11" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="F235" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G235" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B236" s="12" t="inlineStr">
+        <is>
+          <t>13:54:40</t>
+        </is>
+      </c>
+      <c r="C236" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D236" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="E236" s="12" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F236" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G236" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B237" s="11" t="inlineStr">
+        <is>
+          <t>13:59:44</t>
+        </is>
+      </c>
+      <c r="C237" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="D237" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="E237" s="11" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F237" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G237" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H237" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B238" s="12" t="inlineStr">
+        <is>
+          <t>14:04:47</t>
+        </is>
+      </c>
+      <c r="C238" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="D238" s="12" t="n">
+        <v>87</v>
+      </c>
+      <c r="E238" s="12" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F238" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G238" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B239" s="11" t="inlineStr">
+        <is>
+          <t>14:09:52</t>
+        </is>
+      </c>
+      <c r="C239" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D239" s="11" t="n">
+        <v>88</v>
+      </c>
+      <c r="E239" s="11" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F239" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G239" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B240" s="12" t="inlineStr">
+        <is>
+          <t>14:14:56</t>
+        </is>
+      </c>
+      <c r="C240" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="D240" s="12" t="n">
+        <v>91</v>
+      </c>
+      <c r="E240" s="12" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F240" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G240" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B241" s="11" t="inlineStr">
+        <is>
+          <t>14:20:00</t>
+        </is>
+      </c>
+      <c r="C241" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D241" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="E241" s="11" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F241" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G241" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B242" s="12" t="inlineStr">
+        <is>
+          <t>14:25:05</t>
+        </is>
+      </c>
+      <c r="C242" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D242" s="12" t="n">
+        <v>90</v>
+      </c>
+      <c r="E242" s="12" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="F242" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G242" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B243" s="11" t="inlineStr">
+        <is>
+          <t>14:30:08</t>
+        </is>
+      </c>
+      <c r="C243" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="D243" s="11" t="n">
+        <v>91</v>
+      </c>
+      <c r="E243" s="11" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="F243" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G243" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B244" s="12" t="inlineStr">
+        <is>
+          <t>14:35:11</t>
+        </is>
+      </c>
+      <c r="C244" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="D244" s="12" t="n">
+        <v>91</v>
+      </c>
+      <c r="E244" s="12" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="F244" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G244" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H244" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B245" s="11" t="inlineStr">
+        <is>
+          <t>14:40:16</t>
+        </is>
+      </c>
+      <c r="C245" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="D245" s="11" t="n">
+        <v>93</v>
+      </c>
+      <c r="E245" s="11" t="n">
+        <v>66.3</v>
+      </c>
+      <c r="F245" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G245" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H245" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B246" s="12" t="inlineStr">
+        <is>
+          <t>14:45:19</t>
+        </is>
+      </c>
+      <c r="C246" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="D246" s="12" t="n">
+        <v>89</v>
+      </c>
+      <c r="E246" s="12" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="F246" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G246" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H246" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B247" s="11" t="inlineStr">
+        <is>
+          <t>14:50:23</t>
+        </is>
+      </c>
+      <c r="C247" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="D247" s="11" t="n">
+        <v>89</v>
+      </c>
+      <c r="E247" s="11" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="F247" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G247" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H247" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B248" s="12" t="inlineStr">
+        <is>
+          <t>14:55:27</t>
+        </is>
+      </c>
+      <c r="C248" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="D248" s="12" t="n">
+        <v>88</v>
+      </c>
+      <c r="E248" s="12" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="F248" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G248" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B249" s="11" t="inlineStr">
+        <is>
+          <t>15:00:30</t>
+        </is>
+      </c>
+      <c r="C249" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="D249" s="11" t="n">
+        <v>81</v>
+      </c>
+      <c r="E249" s="11" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="F249" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G249" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H249" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B250" s="12" t="inlineStr">
+        <is>
+          <t>15:05:34</t>
+        </is>
+      </c>
+      <c r="C250" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="D250" s="12" t="n">
+        <v>82</v>
+      </c>
+      <c r="E250" s="12" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="F250" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G250" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H250" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B251" s="11" t="inlineStr">
+        <is>
+          <t>15:10:38</t>
+        </is>
+      </c>
+      <c r="C251" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D251" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="E251" s="11" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="F251" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G251" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B252" s="12" t="inlineStr">
+        <is>
+          <t>15:15:43</t>
+        </is>
+      </c>
+      <c r="C252" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="D252" s="12" t="n">
+        <v>82</v>
+      </c>
+      <c r="E252" s="12" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="F252" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G252" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H252" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B253" s="11" t="inlineStr">
+        <is>
+          <t>15:20:47</t>
+        </is>
+      </c>
+      <c r="C253" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D253" s="11" t="n">
+        <v>84</v>
+      </c>
+      <c r="E253" s="11" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="F253" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G253" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B254" s="12" t="inlineStr">
+        <is>
+          <t>15:25:52</t>
+        </is>
+      </c>
+      <c r="C254" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="D254" s="12" t="n">
+        <v>84</v>
+      </c>
+      <c r="E254" s="12" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="F254" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G254" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B255" s="11" t="inlineStr">
+        <is>
+          <t>15:30:56</t>
+        </is>
+      </c>
+      <c r="C255" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="D255" s="11" t="n">
+        <v>84</v>
+      </c>
+      <c r="E255" s="11" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="F255" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G255" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H255" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10088,7 +11082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10630,6 +11624,36 @@
         <v>0</v>
       </c>
       <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>29</v>
+      </c>
+      <c r="C18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-26
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:X36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2350,9 +2350,16 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-26  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A34:X34"/>
@@ -2366,6 +2373,7 @@
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A36:X36"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A22:X22"/>
   </mergeCells>
@@ -11082,7 +11090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11654,6 +11662,36 @@
         <v>0</v>
       </c>
       <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>27</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-29
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:X37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2357,9 +2357,16 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-29  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A34:X34"/>
@@ -2370,6 +2377,7 @@
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A37:X37"/>
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
@@ -11090,7 +11098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11692,6 +11700,36 @@
         <v>0</v>
       </c>
       <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-06-30
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X37"/>
+  <dimension ref="A1:X38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2364,9 +2364,16 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-06-30  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A34:X34"/>
@@ -2375,6 +2382,7 @@
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A32:X32"/>
+    <mergeCell ref="A38:X38"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A37:X37"/>
@@ -2395,7 +2403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H255"/>
+  <dimension ref="A1:H281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11086,6 +11094,890 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B256" s="12" t="inlineStr">
+        <is>
+          <t>13:20:52</t>
+        </is>
+      </c>
+      <c r="C256" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D256" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="E256" s="12" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="F256" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G256" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H256" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B257" s="11" t="inlineStr">
+        <is>
+          <t>13:25:53</t>
+        </is>
+      </c>
+      <c r="C257" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D257" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="E257" s="11" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="F257" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G257" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H257" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B258" s="12" t="inlineStr">
+        <is>
+          <t>13:30:57</t>
+        </is>
+      </c>
+      <c r="C258" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D258" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="E258" s="12" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="F258" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G258" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B259" s="11" t="inlineStr">
+        <is>
+          <t>13:36:00</t>
+        </is>
+      </c>
+      <c r="C259" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D259" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="E259" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="F259" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G259" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H259" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B260" s="12" t="inlineStr">
+        <is>
+          <t>13:41:03</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D260" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="E260" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="F260" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G260" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B261" s="11" t="inlineStr">
+        <is>
+          <t>13:46:06</t>
+        </is>
+      </c>
+      <c r="C261" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D261" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="E261" s="11" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="F261" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G261" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H261" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B262" s="12" t="inlineStr">
+        <is>
+          <t>13:51:10</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D262" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="E262" s="12" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="F262" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G262" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H262" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B263" s="11" t="inlineStr">
+        <is>
+          <t>13:56:14</t>
+        </is>
+      </c>
+      <c r="C263" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D263" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E263" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F263" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G263" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H263" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B264" s="12" t="inlineStr">
+        <is>
+          <t>14:01:17</t>
+        </is>
+      </c>
+      <c r="C264" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D264" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="E264" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F264" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G264" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H264" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B265" s="11" t="inlineStr">
+        <is>
+          <t>14:06:21</t>
+        </is>
+      </c>
+      <c r="C265" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D265" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E265" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F265" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G265" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H265" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B266" s="12" t="inlineStr">
+        <is>
+          <t>14:11:23</t>
+        </is>
+      </c>
+      <c r="C266" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D266" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="E266" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F266" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G266" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B267" s="11" t="inlineStr">
+        <is>
+          <t>14:16:26</t>
+        </is>
+      </c>
+      <c r="C267" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D267" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="E267" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F267" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G267" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B268" s="12" t="inlineStr">
+        <is>
+          <t>14:21:29</t>
+        </is>
+      </c>
+      <c r="C268" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D268" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="E268" s="12" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="F268" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G268" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B269" s="11" t="inlineStr">
+        <is>
+          <t>14:26:32</t>
+        </is>
+      </c>
+      <c r="C269" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D269" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="E269" s="11" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F269" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G269" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B270" s="12" t="inlineStr">
+        <is>
+          <t>14:31:34</t>
+        </is>
+      </c>
+      <c r="C270" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D270" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="E270" s="12" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="F270" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G270" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B271" s="11" t="inlineStr">
+        <is>
+          <t>14:36:37</t>
+        </is>
+      </c>
+      <c r="C271" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D271" s="11" t="n">
+        <v>23</v>
+      </c>
+      <c r="E271" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F271" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G271" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H271" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B272" s="12" t="inlineStr">
+        <is>
+          <t>14:41:40</t>
+        </is>
+      </c>
+      <c r="C272" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D272" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E272" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F272" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G272" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B273" s="11" t="inlineStr">
+        <is>
+          <t>14:46:42</t>
+        </is>
+      </c>
+      <c r="C273" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D273" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="E273" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F273" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G273" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B274" s="12" t="inlineStr">
+        <is>
+          <t>14:51:46</t>
+        </is>
+      </c>
+      <c r="C274" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D274" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="E274" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F274" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G274" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B275" s="11" t="inlineStr">
+        <is>
+          <t>14:56:48</t>
+        </is>
+      </c>
+      <c r="C275" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D275" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="E275" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F275" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G275" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H275" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B276" s="12" t="inlineStr">
+        <is>
+          <t>15:01:50</t>
+        </is>
+      </c>
+      <c r="C276" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D276" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E276" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F276" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G276" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H276" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B277" s="11" t="inlineStr">
+        <is>
+          <t>15:07:12</t>
+        </is>
+      </c>
+      <c r="C277" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D277" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="E277" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F277" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G277" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B278" s="12" t="inlineStr">
+        <is>
+          <t>15:12:15</t>
+        </is>
+      </c>
+      <c r="C278" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D278" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E278" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F278" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G278" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B279" s="11" t="inlineStr">
+        <is>
+          <t>15:17:25</t>
+        </is>
+      </c>
+      <c r="C279" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D279" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="E279" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F279" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G279" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H279" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B280" s="12" t="inlineStr">
+        <is>
+          <t>15:22:28</t>
+        </is>
+      </c>
+      <c r="C280" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D280" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E280" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F280" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G280" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B281" s="11" t="inlineStr">
+        <is>
+          <t>15:27:31</t>
+        </is>
+      </c>
+      <c r="C281" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D281" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="E281" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F281" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G281" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11098,7 +11990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11730,6 +12622,36 @@
         <v>0</v>
       </c>
       <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>26</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-01
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X38"/>
+  <dimension ref="A1:X39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2371,27 +2371,35 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-01  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A37:X37"/>
     <mergeCell ref="A27:X27"/>
-    <mergeCell ref="A30:X30"/>
-    <mergeCell ref="A34:X34"/>
+    <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A33:X33"/>
+    <mergeCell ref="A23:X23"/>
+    <mergeCell ref="A32:X32"/>
+    <mergeCell ref="A22:X22"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A35:X35"/>
-    <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A38:X38"/>
+    <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A31:X31"/>
+    <mergeCell ref="A30:X30"/>
+    <mergeCell ref="A39:X39"/>
+    <mergeCell ref="A34:X34"/>
     <mergeCell ref="A24:X24"/>
-    <mergeCell ref="A32:X32"/>
-    <mergeCell ref="A38:X38"/>
-    <mergeCell ref="A25:X25"/>
-    <mergeCell ref="A28:X28"/>
-    <mergeCell ref="A37:X37"/>
-    <mergeCell ref="A33:X33"/>
-    <mergeCell ref="A23:X23"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
-    <mergeCell ref="A31:X31"/>
-    <mergeCell ref="A22:X22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11990,7 +11998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12652,6 +12660,36 @@
         <v>0</v>
       </c>
       <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-02
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X39"/>
+  <dimension ref="A1:X40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2378,9 +2378,16 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-02  End of Day  |  Signals: 5  |  Stocks: KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A27:X27"/>
@@ -2394,6 +2401,7 @@
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A31:X31"/>
+    <mergeCell ref="A40:X40"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
@@ -2411,7 +2419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H281"/>
+  <dimension ref="A1:H311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11986,6 +11994,1026 @@
         </is>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B282" s="12" t="inlineStr">
+        <is>
+          <t>12:57:27</t>
+        </is>
+      </c>
+      <c r="C282" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D282" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="E282" s="12" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="F282" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G282" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B283" s="11" t="inlineStr">
+        <is>
+          <t>13:02:29</t>
+        </is>
+      </c>
+      <c r="C283" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D283" s="11" t="n">
+        <v>173</v>
+      </c>
+      <c r="E283" s="11" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F283" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G283" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H283" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B284" s="12" t="inlineStr">
+        <is>
+          <t>13:07:32</t>
+        </is>
+      </c>
+      <c r="C284" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D284" s="12" t="n">
+        <v>173</v>
+      </c>
+      <c r="E284" s="12" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="F284" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G284" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B285" s="11" t="inlineStr">
+        <is>
+          <t>13:12:44</t>
+        </is>
+      </c>
+      <c r="C285" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D285" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="E285" s="11" t="n">
+        <v>48</v>
+      </c>
+      <c r="F285" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G285" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H285" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B286" s="12" t="inlineStr">
+        <is>
+          <t>13:17:47</t>
+        </is>
+      </c>
+      <c r="C286" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D286" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="E286" s="12" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="F286" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G286" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H286" s="12" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B287" s="11" t="inlineStr">
+        <is>
+          <t>13:22:59</t>
+        </is>
+      </c>
+      <c r="C287" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D287" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="E287" s="11" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="F287" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G287" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H287" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B288" s="12" t="inlineStr">
+        <is>
+          <t>13:28:21</t>
+        </is>
+      </c>
+      <c r="C288" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D288" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="E288" s="12" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="F288" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G288" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H288" s="12" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B289" s="11" t="inlineStr">
+        <is>
+          <t>13:33:24</t>
+        </is>
+      </c>
+      <c r="C289" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D289" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="E289" s="11" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="F289" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G289" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H289" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B290" s="12" t="inlineStr">
+        <is>
+          <t>13:38:34</t>
+        </is>
+      </c>
+      <c r="C290" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D290" s="12" t="n">
+        <v>172</v>
+      </c>
+      <c r="E290" s="12" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="F290" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G290" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H290" s="12" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B291" s="11" t="inlineStr">
+        <is>
+          <t>13:43:46</t>
+        </is>
+      </c>
+      <c r="C291" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D291" s="11" t="n">
+        <v>171</v>
+      </c>
+      <c r="E291" s="11" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="F291" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G291" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H291" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B292" s="12" t="inlineStr">
+        <is>
+          <t>13:48:49</t>
+        </is>
+      </c>
+      <c r="C292" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D292" s="12" t="n">
+        <v>173</v>
+      </c>
+      <c r="E292" s="12" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="F292" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G292" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H292" s="12" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B293" s="11" t="inlineStr">
+        <is>
+          <t>13:53:53</t>
+        </is>
+      </c>
+      <c r="C293" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D293" s="11" t="n">
+        <v>173</v>
+      </c>
+      <c r="E293" s="11" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F293" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G293" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H293" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B294" s="12" t="inlineStr">
+        <is>
+          <t>13:59:16</t>
+        </is>
+      </c>
+      <c r="C294" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D294" s="12" t="n">
+        <v>174</v>
+      </c>
+      <c r="E294" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="F294" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G294" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H294" s="12" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B295" s="11" t="inlineStr">
+        <is>
+          <t>14:04:20</t>
+        </is>
+      </c>
+      <c r="C295" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D295" s="11" t="n">
+        <v>173</v>
+      </c>
+      <c r="E295" s="11" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="F295" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G295" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H295" s="11" t="inlineStr">
+        <is>
+          <t>BSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B296" s="12" t="inlineStr">
+        <is>
+          <t>14:09:24</t>
+        </is>
+      </c>
+      <c r="C296" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D296" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="E296" s="12" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="F296" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G296" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H296" s="12" t="inlineStr">
+        <is>
+          <t>BSE, GODFRYPHLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B297" s="11" t="inlineStr">
+        <is>
+          <t>14:14:36</t>
+        </is>
+      </c>
+      <c r="C297" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D297" s="11" t="n">
+        <v>177</v>
+      </c>
+      <c r="E297" s="11" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="F297" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G297" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H297" s="11" t="inlineStr">
+        <is>
+          <t>BSE, GODFRYPHLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B298" s="12" t="inlineStr">
+        <is>
+          <t>14:19:39</t>
+        </is>
+      </c>
+      <c r="C298" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D298" s="12" t="n">
+        <v>178</v>
+      </c>
+      <c r="E298" s="12" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="F298" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G298" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H298" s="12" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B299" s="11" t="inlineStr">
+        <is>
+          <t>14:24:43</t>
+        </is>
+      </c>
+      <c r="C299" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D299" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="E299" s="11" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F299" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G299" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H299" s="11" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B300" s="12" t="inlineStr">
+        <is>
+          <t>14:29:48</t>
+        </is>
+      </c>
+      <c r="C300" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D300" s="12" t="n">
+        <v>178</v>
+      </c>
+      <c r="E300" s="12" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="F300" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G300" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H300" s="12" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B301" s="11" t="inlineStr">
+        <is>
+          <t>14:34:52</t>
+        </is>
+      </c>
+      <c r="C301" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D301" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="E301" s="11" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="F301" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G301" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H301" s="11" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B302" s="12" t="inlineStr">
+        <is>
+          <t>14:40:03</t>
+        </is>
+      </c>
+      <c r="C302" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D302" s="12" t="n">
+        <v>178</v>
+      </c>
+      <c r="E302" s="12" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F302" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G302" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H302" s="12" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B303" s="11" t="inlineStr">
+        <is>
+          <t>14:45:16</t>
+        </is>
+      </c>
+      <c r="C303" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D303" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="E303" s="11" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="F303" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G303" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H303" s="11" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B304" s="12" t="inlineStr">
+        <is>
+          <t>14:50:20</t>
+        </is>
+      </c>
+      <c r="C304" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D304" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="E304" s="12" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F304" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G304" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H304" s="12" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B305" s="11" t="inlineStr">
+        <is>
+          <t>14:55:23</t>
+        </is>
+      </c>
+      <c r="C305" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D305" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="E305" s="11" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="F305" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G305" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H305" s="11" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B306" s="12" t="inlineStr">
+        <is>
+          <t>15:00:27</t>
+        </is>
+      </c>
+      <c r="C306" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D306" s="12" t="n">
+        <v>176</v>
+      </c>
+      <c r="E306" s="12" t="n">
+        <v>52</v>
+      </c>
+      <c r="F306" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G306" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H306" s="12" t="inlineStr">
+        <is>
+          <t>BSE, BANKBARODA, GODFRYPHLP, SONACOMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B307" s="11" t="inlineStr">
+        <is>
+          <t>15:05:30</t>
+        </is>
+      </c>
+      <c r="C307" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D307" s="11" t="n">
+        <v>177</v>
+      </c>
+      <c r="E307" s="11" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="F307" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G307" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H307" s="11" t="inlineStr">
+        <is>
+          <t>KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B308" s="12" t="inlineStr">
+        <is>
+          <t>15:10:34</t>
+        </is>
+      </c>
+      <c r="C308" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="D308" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="E308" s="12" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="F308" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G308" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H308" s="12" t="inlineStr">
+        <is>
+          <t>KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B309" s="11" t="inlineStr">
+        <is>
+          <t>15:15:50</t>
+        </is>
+      </c>
+      <c r="C309" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D309" s="11" t="n">
+        <v>178</v>
+      </c>
+      <c r="E309" s="11" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F309" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G309" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H309" s="11" t="inlineStr">
+        <is>
+          <t>KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B310" s="12" t="inlineStr">
+        <is>
+          <t>15:20:53</t>
+        </is>
+      </c>
+      <c r="C310" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D310" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="E310" s="12" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="F310" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G310" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H310" s="12" t="inlineStr">
+        <is>
+          <t>KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B311" s="11" t="inlineStr">
+        <is>
+          <t>15:25:57</t>
+        </is>
+      </c>
+      <c r="C311" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D311" s="11" t="n">
+        <v>183</v>
+      </c>
+      <c r="E311" s="11" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="F311" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G311" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H311" s="11" t="inlineStr">
+        <is>
+          <t>KFINTECH, GODFRYPHLP, SONACOMS, BSE, BANKBARODA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11998,7 +13026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12690,6 +13718,36 @@
         <v>0</v>
       </c>
       <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="C23" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-07-03 06:49 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -13764,7 +13764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14396,6 +14396,225 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>POLICYBZR</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="M9" s="24" t="inlineStr"/>
+      <c r="N9" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O9" s="24" t="n">
+        <v>25.25</v>
+      </c>
+      <c r="P9" s="24" t="n">
+        <v>482.2</v>
+      </c>
+      <c r="Q9" s="24" t="n">
+        <v>1595</v>
+      </c>
+      <c r="R9" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S9" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="M10" s="24" t="inlineStr"/>
+      <c r="N10" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O10" s="24" t="n">
+        <v>18.53</v>
+      </c>
+      <c r="P10" s="24" t="n">
+        <v>184.1</v>
+      </c>
+      <c r="Q10" s="24" t="n">
+        <v>896.6</v>
+      </c>
+      <c r="R10" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S10" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>ALKEM</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="22" t="n">
+        <v>68.08</v>
+      </c>
+      <c r="M11" s="22" t="inlineStr"/>
+      <c r="N11" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O11" s="22" t="n">
+        <v>14.52</v>
+      </c>
+      <c r="P11" s="22" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="Q11" s="22" t="n">
+        <v>5596</v>
+      </c>
+      <c r="R11" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-03
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X40"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2385,10 +2385,18 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-03  End of Day  |  Signals: 9  |  Stocks: MCX, POWERINDIA, KALYANKJIL, KAYNES, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A26:X26"/>
@@ -2419,7 +2427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H311"/>
+  <dimension ref="A1:H347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13014,6 +13022,1230 @@
         </is>
       </c>
     </row>
+    <row r="312">
+      <c r="A312" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B312" s="12" t="inlineStr">
+        <is>
+          <t>12:28:27</t>
+        </is>
+      </c>
+      <c r="C312" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D312" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="E312" s="12" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="F312" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G312" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H312" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B313" s="11" t="inlineStr">
+        <is>
+          <t>12:33:31</t>
+        </is>
+      </c>
+      <c r="C313" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D313" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="E313" s="11" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F313" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G313" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B314" s="12" t="inlineStr">
+        <is>
+          <t>12:38:36</t>
+        </is>
+      </c>
+      <c r="C314" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D314" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="E314" s="12" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F314" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G314" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B315" s="11" t="inlineStr">
+        <is>
+          <t>12:43:41</t>
+        </is>
+      </c>
+      <c r="C315" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D315" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E315" s="11" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="F315" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G315" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H315" s="11" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B316" s="12" t="inlineStr">
+        <is>
+          <t>12:48:47</t>
+        </is>
+      </c>
+      <c r="C316" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D316" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E316" s="12" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="F316" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G316" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H316" s="12" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B317" s="11" t="inlineStr">
+        <is>
+          <t>12:53:51</t>
+        </is>
+      </c>
+      <c r="C317" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D317" s="11" t="n">
+        <v>169</v>
+      </c>
+      <c r="E317" s="11" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="F317" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G317" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H317" s="11" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B318" s="12" t="inlineStr">
+        <is>
+          <t>12:58:58</t>
+        </is>
+      </c>
+      <c r="C318" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D318" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E318" s="12" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="F318" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G318" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H318" s="12" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B319" s="11" t="inlineStr">
+        <is>
+          <t>13:04:03</t>
+        </is>
+      </c>
+      <c r="C319" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D319" s="11" t="n">
+        <v>169</v>
+      </c>
+      <c r="E319" s="11" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="F319" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G319" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H319" s="11" t="inlineStr">
+        <is>
+          <t>NUVAMA, PERSISTENT, MANKIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B320" s="12" t="inlineStr">
+        <is>
+          <t>13:09:08</t>
+        </is>
+      </c>
+      <c r="C320" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D320" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="E320" s="12" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="F320" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G320" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H320" s="12" t="inlineStr">
+        <is>
+          <t>NUVAMA, TIINDIA, PERSISTENT, MANKIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B321" s="11" t="inlineStr">
+        <is>
+          <t>13:14:14</t>
+        </is>
+      </c>
+      <c r="C321" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D321" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E321" s="11" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="F321" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G321" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H321" s="11" t="inlineStr">
+        <is>
+          <t>NUVAMA, TIINDIA, PERSISTENT, MANKIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B322" s="12" t="inlineStr">
+        <is>
+          <t>13:19:19</t>
+        </is>
+      </c>
+      <c r="C322" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D322" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="E322" s="12" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="F322" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G322" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H322" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B323" s="11" t="inlineStr">
+        <is>
+          <t>13:24:23</t>
+        </is>
+      </c>
+      <c r="C323" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D323" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E323" s="11" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="F323" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G323" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H323" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B324" s="12" t="inlineStr">
+        <is>
+          <t>13:29:29</t>
+        </is>
+      </c>
+      <c r="C324" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D324" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E324" s="12" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="F324" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G324" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H324" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B325" s="11" t="inlineStr">
+        <is>
+          <t>13:34:34</t>
+        </is>
+      </c>
+      <c r="C325" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D325" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="E325" s="11" t="n">
+        <v>53</v>
+      </c>
+      <c r="F325" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G325" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H325" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B326" s="12" t="inlineStr">
+        <is>
+          <t>13:39:39</t>
+        </is>
+      </c>
+      <c r="C326" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D326" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E326" s="12" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="F326" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G326" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H326" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B327" s="11" t="inlineStr">
+        <is>
+          <t>13:44:44</t>
+        </is>
+      </c>
+      <c r="C327" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D327" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E327" s="11" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="F327" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G327" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H327" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B328" s="12" t="inlineStr">
+        <is>
+          <t>13:49:49</t>
+        </is>
+      </c>
+      <c r="C328" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D328" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="E328" s="12" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="F328" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G328" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H328" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B329" s="11" t="inlineStr">
+        <is>
+          <t>13:54:53</t>
+        </is>
+      </c>
+      <c r="C329" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D329" s="11" t="n">
+        <v>166</v>
+      </c>
+      <c r="E329" s="11" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="F329" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G329" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H329" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B330" s="12" t="inlineStr">
+        <is>
+          <t>14:00:07</t>
+        </is>
+      </c>
+      <c r="C330" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D330" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="E330" s="12" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="F330" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G330" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H330" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B331" s="11" t="inlineStr">
+        <is>
+          <t>14:05:11</t>
+        </is>
+      </c>
+      <c r="C331" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D331" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E331" s="11" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="F331" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G331" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H331" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B332" s="12" t="inlineStr">
+        <is>
+          <t>14:10:16</t>
+        </is>
+      </c>
+      <c r="C332" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D332" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="E332" s="12" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="F332" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G332" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H332" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B333" s="11" t="inlineStr">
+        <is>
+          <t>14:15:22</t>
+        </is>
+      </c>
+      <c r="C333" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D333" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="E333" s="11" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="F333" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G333" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H333" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B334" s="12" t="inlineStr">
+        <is>
+          <t>14:20:26</t>
+        </is>
+      </c>
+      <c r="C334" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D334" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="E334" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="F334" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G334" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H334" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B335" s="11" t="inlineStr">
+        <is>
+          <t>14:25:31</t>
+        </is>
+      </c>
+      <c r="C335" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D335" s="11" t="n">
+        <v>169</v>
+      </c>
+      <c r="E335" s="11" t="n">
+        <v>54</v>
+      </c>
+      <c r="F335" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G335" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H335" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B336" s="12" t="inlineStr">
+        <is>
+          <t>14:30:37</t>
+        </is>
+      </c>
+      <c r="C336" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D336" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="E336" s="12" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="F336" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G336" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H336" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B337" s="11" t="inlineStr">
+        <is>
+          <t>14:35:41</t>
+        </is>
+      </c>
+      <c r="C337" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D337" s="11" t="n">
+        <v>167</v>
+      </c>
+      <c r="E337" s="11" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="F337" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G337" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H337" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B338" s="12" t="inlineStr">
+        <is>
+          <t>14:40:46</t>
+        </is>
+      </c>
+      <c r="C338" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="D338" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="E338" s="12" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F338" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G338" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H338" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B339" s="11" t="inlineStr">
+        <is>
+          <t>14:45:52</t>
+        </is>
+      </c>
+      <c r="C339" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D339" s="11" t="n">
+        <v>170</v>
+      </c>
+      <c r="E339" s="11" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F339" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G339" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H339" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B340" s="12" t="inlineStr">
+        <is>
+          <t>14:50:57</t>
+        </is>
+      </c>
+      <c r="C340" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D340" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="E340" s="12" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="F340" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G340" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="H340" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B341" s="11" t="inlineStr">
+        <is>
+          <t>14:56:03</t>
+        </is>
+      </c>
+      <c r="C341" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D341" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="E341" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="F341" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G341" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H341" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B342" s="12" t="inlineStr">
+        <is>
+          <t>15:01:09</t>
+        </is>
+      </c>
+      <c r="C342" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D342" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="E342" s="12" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="F342" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G342" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H342" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, KALYANKJIL, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B343" s="11" t="inlineStr">
+        <is>
+          <t>15:06:14</t>
+        </is>
+      </c>
+      <c r="C343" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D343" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="E343" s="11" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="F343" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G343" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H343" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, KALYANKJIL, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B344" s="12" t="inlineStr">
+        <is>
+          <t>15:11:18</t>
+        </is>
+      </c>
+      <c r="C344" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D344" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="E344" s="12" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="F344" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G344" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H344" s="12" t="inlineStr">
+        <is>
+          <t>POWERINDIA, KALYANKJIL, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B345" s="11" t="inlineStr">
+        <is>
+          <t>15:16:24</t>
+        </is>
+      </c>
+      <c r="C345" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="D345" s="11" t="n">
+        <v>166</v>
+      </c>
+      <c r="E345" s="11" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="F345" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G345" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H345" s="11" t="inlineStr">
+        <is>
+          <t>POWERINDIA, KALYANKJIL, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B346" s="12" t="inlineStr">
+        <is>
+          <t>15:21:29</t>
+        </is>
+      </c>
+      <c r="C346" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="D346" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="E346" s="12" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="F346" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G346" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="H346" s="12" t="inlineStr">
+        <is>
+          <t>MCX, POWERINDIA, KALYANKJIL, KAYNES, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B347" s="11" t="inlineStr">
+        <is>
+          <t>15:26:34</t>
+        </is>
+      </c>
+      <c r="C347" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="D347" s="11" t="n">
+        <v>169</v>
+      </c>
+      <c r="E347" s="11" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="F347" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G347" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H347" s="11" t="inlineStr">
+        <is>
+          <t>MCX, POWERINDIA, KALYANKJIL, KAYNES, PERSISTENT, MANKIND, RBLBANK, NUVAMA, TIINDIA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13026,7 +14258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13748,6 +14980,36 @@
         <v>0</v>
       </c>
       <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="D24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-06
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X41"/>
+  <dimension ref="A1:X42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2392,14 +2392,22 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-06  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A42:X42"/>
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
@@ -14258,7 +14266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15010,6 +15018,36 @@
         <v>0</v>
       </c>
       <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B25" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-07-07 07:02 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -15064,7 +15064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15915,6 +15915,225 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="M12" s="24" t="inlineStr"/>
+      <c r="N12" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O12" s="24" t="n">
+        <v>31.41</v>
+      </c>
+      <c r="P12" s="24" t="n">
+        <v>1835.8</v>
+      </c>
+      <c r="Q12" s="24" t="n">
+        <v>2933.8</v>
+      </c>
+      <c r="R12" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S12" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>COCHINSHIP</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K13" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="24" t="n">
+        <v>51.72</v>
+      </c>
+      <c r="M13" s="24" t="inlineStr"/>
+      <c r="N13" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O13" s="24" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="P13" s="24" t="n">
+        <v>138.5</v>
+      </c>
+      <c r="Q13" s="24" t="n">
+        <v>1453.5</v>
+      </c>
+      <c r="R13" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>NAUKRI</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="22" t="n">
+        <v>38.23999999999999</v>
+      </c>
+      <c r="M14" s="22" t="inlineStr"/>
+      <c r="N14" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O14" s="22" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="P14" s="22" t="n">
+        <v>361.7</v>
+      </c>
+      <c r="Q14" s="22" t="n">
+        <v>1130</v>
+      </c>
+      <c r="R14" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-07
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X42"/>
+  <dimension ref="A1:X43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2399,9 +2399,16 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-07  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2414,6 +2421,7 @@
     <mergeCell ref="A22:X22"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A35:X35"/>
+    <mergeCell ref="A43:X43"/>
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A31:X31"/>
@@ -14266,7 +14274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15048,6 +15056,36 @@
         <v>0</v>
       </c>
       <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="C26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-08
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X43"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2406,9 +2406,16 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-08  End of Day  |  Signals: 30  |  Stocks: NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, ABCAPITAL, PNB, MAXHEALTH, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, BANKBARODA, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, HDFCBANK, AXISBANK  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2425,6 +2432,7 @@
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A31:X31"/>
+    <mergeCell ref="A44:X44"/>
     <mergeCell ref="A40:X40"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
@@ -2443,7 +2451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H347"/>
+  <dimension ref="A1:H383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14262,6 +14270,1230 @@
         </is>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B348" s="12" t="inlineStr">
+        <is>
+          <t>11:54:43</t>
+        </is>
+      </c>
+      <c r="C348" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D348" s="12" t="n">
+        <v>155</v>
+      </c>
+      <c r="E348" s="12" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="F348" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G348" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B349" s="11" t="inlineStr">
+        <is>
+          <t>11:59:45</t>
+        </is>
+      </c>
+      <c r="C349" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D349" s="11" t="n">
+        <v>152</v>
+      </c>
+      <c r="E349" s="11" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="F349" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G349" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H349" s="11" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B350" s="12" t="inlineStr">
+        <is>
+          <t>12:04:47</t>
+        </is>
+      </c>
+      <c r="C350" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D350" s="12" t="n">
+        <v>153</v>
+      </c>
+      <c r="E350" s="12" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="F350" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G350" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H350" s="12" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B351" s="11" t="inlineStr">
+        <is>
+          <t>12:09:50</t>
+        </is>
+      </c>
+      <c r="C351" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D351" s="11" t="n">
+        <v>154</v>
+      </c>
+      <c r="E351" s="11" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F351" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G351" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H351" s="11" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B352" s="12" t="inlineStr">
+        <is>
+          <t>12:14:53</t>
+        </is>
+      </c>
+      <c r="C352" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D352" s="12" t="n">
+        <v>155</v>
+      </c>
+      <c r="E352" s="12" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F352" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G352" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H352" s="12" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B353" s="11" t="inlineStr">
+        <is>
+          <t>12:19:55</t>
+        </is>
+      </c>
+      <c r="C353" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D353" s="11" t="n">
+        <v>156</v>
+      </c>
+      <c r="E353" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F353" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G353" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H353" s="11" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B354" s="12" t="inlineStr">
+        <is>
+          <t>12:24:59</t>
+        </is>
+      </c>
+      <c r="C354" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D354" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E354" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F354" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G354" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H354" s="12" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B355" s="11" t="inlineStr">
+        <is>
+          <t>12:30:02</t>
+        </is>
+      </c>
+      <c r="C355" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D355" s="11" t="n">
+        <v>158</v>
+      </c>
+      <c r="E355" s="11" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="F355" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G355" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H355" s="11" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B356" s="12" t="inlineStr">
+        <is>
+          <t>12:35:04</t>
+        </is>
+      </c>
+      <c r="C356" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D356" s="12" t="n">
+        <v>159</v>
+      </c>
+      <c r="E356" s="12" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="F356" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G356" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H356" s="12" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B357" s="11" t="inlineStr">
+        <is>
+          <t>12:40:08</t>
+        </is>
+      </c>
+      <c r="C357" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D357" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E357" s="11" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="F357" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G357" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H357" s="11" t="inlineStr">
+        <is>
+          <t>360ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B358" s="12" t="inlineStr">
+        <is>
+          <t>12:45:10</t>
+        </is>
+      </c>
+      <c r="C358" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D358" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="E358" s="12" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="F358" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G358" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H358" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B359" s="11" t="inlineStr">
+        <is>
+          <t>12:50:13</t>
+        </is>
+      </c>
+      <c r="C359" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D359" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E359" s="11" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="F359" s="11" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G359" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H359" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B360" s="12" t="inlineStr">
+        <is>
+          <t>12:55:16</t>
+        </is>
+      </c>
+      <c r="C360" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D360" s="12" t="n">
+        <v>159</v>
+      </c>
+      <c r="E360" s="12" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F360" s="12" t="inlineStr">
+        <is>
+          <t>Midday Lull</t>
+        </is>
+      </c>
+      <c r="G360" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H360" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B361" s="11" t="inlineStr">
+        <is>
+          <t>13:00:18</t>
+        </is>
+      </c>
+      <c r="C361" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D361" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E361" s="11" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="F361" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G361" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H361" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B362" s="12" t="inlineStr">
+        <is>
+          <t>13:05:21</t>
+        </is>
+      </c>
+      <c r="C362" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D362" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E362" s="12" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="F362" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G362" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H362" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B363" s="11" t="inlineStr">
+        <is>
+          <t>13:10:25</t>
+        </is>
+      </c>
+      <c r="C363" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D363" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E363" s="11" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="F363" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G363" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H363" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B364" s="12" t="inlineStr">
+        <is>
+          <t>13:15:27</t>
+        </is>
+      </c>
+      <c r="C364" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D364" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="E364" s="12" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="F364" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G364" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H364" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B365" s="11" t="inlineStr">
+        <is>
+          <t>13:20:30</t>
+        </is>
+      </c>
+      <c r="C365" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D365" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E365" s="11" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="F365" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G365" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H365" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B366" s="12" t="inlineStr">
+        <is>
+          <t>13:25:33</t>
+        </is>
+      </c>
+      <c r="C366" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D366" s="12" t="n">
+        <v>157</v>
+      </c>
+      <c r="E366" s="12" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="F366" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G366" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H366" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B367" s="11" t="inlineStr">
+        <is>
+          <t>13:30:36</t>
+        </is>
+      </c>
+      <c r="C367" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D367" s="11" t="n">
+        <v>158</v>
+      </c>
+      <c r="E367" s="11" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="F367" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G367" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H367" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D, IEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B368" s="12" t="inlineStr">
+        <is>
+          <t>13:35:39</t>
+        </is>
+      </c>
+      <c r="C368" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D368" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="E368" s="12" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="F368" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G368" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H368" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D, IEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B369" s="11" t="inlineStr">
+        <is>
+          <t>13:40:43</t>
+        </is>
+      </c>
+      <c r="C369" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D369" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E369" s="11" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="F369" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G369" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H369" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D, IEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B370" s="12" t="inlineStr">
+        <is>
+          <t>13:45:45</t>
+        </is>
+      </c>
+      <c r="C370" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D370" s="12" t="n">
+        <v>164</v>
+      </c>
+      <c r="E370" s="12" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="F370" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G370" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H370" s="12" t="inlineStr">
+        <is>
+          <t>360ONE, KALYANKJIL, GVT&amp;D, IEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B371" s="11" t="inlineStr">
+        <is>
+          <t>13:50:49</t>
+        </is>
+      </c>
+      <c r="C371" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D371" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E371" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="F371" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G371" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H371" s="11" t="inlineStr">
+        <is>
+          <t>360ONE, IEX, LODHA, KALYANKJIL, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B372" s="12" t="inlineStr">
+        <is>
+          <t>13:55:53</t>
+        </is>
+      </c>
+      <c r="C372" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D372" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="E372" s="12" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="F372" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G372" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="H372" s="12" t="inlineStr">
+        <is>
+          <t>PNB, 360ONE, BAJAJHLDNG, GMRAIRPORT, IEX, NBCC, LODHA, CROMPTON, HDFCAMC, AMBER, KALYANKJIL, CONCOR, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B373" s="11" t="inlineStr">
+        <is>
+          <t>14:00:56</t>
+        </is>
+      </c>
+      <c r="C373" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D373" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="E373" s="11" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="F373" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G373" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H373" s="11" t="inlineStr">
+        <is>
+          <t>PNB, 360ONE, BAJAJHLDNG, GMRAIRPORT, PNBHOUSING, IEX, NBCC, LODHA, CROMPTON, HDFCAMC, AMBER, FORCEMOT, CAMS, KALYANKJIL, CONCOR, GVT&amp;D</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B374" s="12" t="inlineStr">
+        <is>
+          <t>14:05:58</t>
+        </is>
+      </c>
+      <c r="C374" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="D374" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="E374" s="12" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="F374" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G374" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H374" s="12" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, PNBHOUSING, CAMS, PNB, IEX, AMBER, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, BAJAJHLDNG, LODHA, HDFCAMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B375" s="11" t="inlineStr">
+        <is>
+          <t>14:11:04</t>
+        </is>
+      </c>
+      <c r="C375" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D375" s="11" t="n">
+        <v>169</v>
+      </c>
+      <c r="E375" s="11" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="F375" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G375" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="H375" s="11" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, PNBHOUSING, CAMS, PNB, IEX, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, BAJAJHLDNG, LODHA, HDFCAMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B376" s="12" t="inlineStr">
+        <is>
+          <t>14:16:09</t>
+        </is>
+      </c>
+      <c r="C376" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D376" s="12" t="n">
+        <v>161</v>
+      </c>
+      <c r="E376" s="12" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="F376" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G376" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="H376" s="12" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B377" s="11" t="inlineStr">
+        <is>
+          <t>14:21:13</t>
+        </is>
+      </c>
+      <c r="C377" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D377" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E377" s="11" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F377" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G377" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="H377" s="11" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B378" s="12" t="inlineStr">
+        <is>
+          <t>14:26:17</t>
+        </is>
+      </c>
+      <c r="C378" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="D378" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E378" s="12" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F378" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G378" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="H378" s="12" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B379" s="11" t="inlineStr">
+        <is>
+          <t>14:31:20</t>
+        </is>
+      </c>
+      <c r="C379" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D379" s="11" t="n">
+        <v>156</v>
+      </c>
+      <c r="E379" s="11" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="F379" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G379" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="H379" s="11" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B380" s="12" t="inlineStr">
+        <is>
+          <t>14:36:24</t>
+        </is>
+      </c>
+      <c r="C380" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="D380" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E380" s="12" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="F380" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G380" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="H380" s="12" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, MAXHEALTH, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, BANKBARODA, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B381" s="11" t="inlineStr">
+        <is>
+          <t>14:41:28</t>
+        </is>
+      </c>
+      <c r="C381" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="D381" s="11" t="n">
+        <v>159</v>
+      </c>
+      <c r="E381" s="11" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="F381" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G381" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="H381" s="11" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, MAXHEALTH, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, BANKBARODA, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, HDFCBANK, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B382" s="12" t="inlineStr">
+        <is>
+          <t>14:46:32</t>
+        </is>
+      </c>
+      <c r="C382" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="D382" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E382" s="12" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="F382" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G382" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="H382" s="12" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, PNB, MAXHEALTH, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, BANKBARODA, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, HDFCBANK, AXISBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B383" s="11" t="inlineStr">
+        <is>
+          <t>14:51:37</t>
+        </is>
+      </c>
+      <c r="C383" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="D383" s="11" t="n">
+        <v>156</v>
+      </c>
+      <c r="E383" s="11" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="F383" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G383" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H383" s="11" t="inlineStr">
+        <is>
+          <t>NBCC, CROMPTON, M&amp;M, PNBHOUSING, CAMS, ABCAPITAL, PNB, MAXHEALTH, IEX, UPL, AMBER, ASIANPAINT, MOTHERSON, KALYANKJIL, FINNIFTY, 360ONE, GMRAIRPORT, FORCEMOT, BANKBARODA, CONCOR, CHOLAFIN, JUBLFOOD, GVT&amp;D, SWIGGY, BAJAJHLDNG, LODHA, HDFCAMC, SUZLON, HDFCBANK, AXISBANK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14274,7 +15506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15086,6 +16318,36 @@
         <v>0</v>
       </c>
       <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B27" s="19" t="n">
+        <v>36</v>
+      </c>
+      <c r="C27" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="D27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-09
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X44"/>
+  <dimension ref="A1:X45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2413,9 +2413,16 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-09  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="24">
+  <mergeCells count="25">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2438,6 +2445,7 @@
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A45:X45"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
   </mergeCells>
@@ -15506,7 +15514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16348,6 +16356,36 @@
         <v>0</v>
       </c>
       <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="C28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-07-10 07:02 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -16402,7 +16402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S14"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17472,6 +17472,152 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>CDSL</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="22" t="n">
+        <v>80</v>
+      </c>
+      <c r="M15" s="22" t="inlineStr"/>
+      <c r="N15" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O15" s="22" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="P15" s="22" t="n">
+        <v>242.7</v>
+      </c>
+      <c r="Q15" s="22" t="n">
+        <v>1418.9</v>
+      </c>
+      <c r="R15" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S15" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="22" t="n">
+        <v>30.44</v>
+      </c>
+      <c r="M16" s="22" t="inlineStr"/>
+      <c r="N16" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O16" s="22" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="P16" s="22" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="Q16" s="22" t="n">
+        <v>11637</v>
+      </c>
+      <c r="R16" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S16" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-10
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X45"/>
+  <dimension ref="A1:X46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2420,12 +2420,20 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-10  End of Day  |  Signals: 8  |  Stocks: PAYTM, UNIONBANK, PNB, INDIANB, TMPV, KALYANKJIL, CDSL, NUVAMA  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="25">
+  <mergeCells count="26">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
+    <mergeCell ref="A46:X46"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A42:X42"/>
@@ -2459,7 +2467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H383"/>
+  <dimension ref="A1:H413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15502,6 +15510,1026 @@
         </is>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B384" s="12" t="inlineStr">
+        <is>
+          <t>13:01:56</t>
+        </is>
+      </c>
+      <c r="C384" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D384" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="E384" s="12" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="F384" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G384" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H384" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B385" s="11" t="inlineStr">
+        <is>
+          <t>13:06:58</t>
+        </is>
+      </c>
+      <c r="C385" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D385" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="E385" s="11" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="F385" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G385" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H385" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B386" s="12" t="inlineStr">
+        <is>
+          <t>13:12:02</t>
+        </is>
+      </c>
+      <c r="C386" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D386" s="12" t="n">
+        <v>161</v>
+      </c>
+      <c r="E386" s="12" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="F386" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G386" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H386" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B387" s="11" t="inlineStr">
+        <is>
+          <t>13:17:06</t>
+        </is>
+      </c>
+      <c r="C387" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D387" s="11" t="n">
+        <v>161</v>
+      </c>
+      <c r="E387" s="11" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="F387" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G387" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H387" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B388" s="12" t="inlineStr">
+        <is>
+          <t>13:22:09</t>
+        </is>
+      </c>
+      <c r="C388" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D388" s="12" t="n">
+        <v>161</v>
+      </c>
+      <c r="E388" s="12" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="F388" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G388" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H388" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B389" s="11" t="inlineStr">
+        <is>
+          <t>13:27:12</t>
+        </is>
+      </c>
+      <c r="C389" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D389" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="E389" s="11" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="F389" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G389" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H389" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B390" s="12" t="inlineStr">
+        <is>
+          <t>13:32:16</t>
+        </is>
+      </c>
+      <c r="C390" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D390" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="E390" s="12" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="F390" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G390" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H390" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B391" s="11" t="inlineStr">
+        <is>
+          <t>13:37:19</t>
+        </is>
+      </c>
+      <c r="C391" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D391" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="E391" s="11" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="F391" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G391" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H391" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B392" s="12" t="inlineStr">
+        <is>
+          <t>13:42:22</t>
+        </is>
+      </c>
+      <c r="C392" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D392" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E392" s="12" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="F392" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G392" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H392" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B393" s="11" t="inlineStr">
+        <is>
+          <t>13:47:26</t>
+        </is>
+      </c>
+      <c r="C393" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D393" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="E393" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="F393" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G393" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H393" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B394" s="12" t="inlineStr">
+        <is>
+          <t>13:52:29</t>
+        </is>
+      </c>
+      <c r="C394" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D394" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="E394" s="12" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F394" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G394" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H394" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B395" s="11" t="inlineStr">
+        <is>
+          <t>13:57:34</t>
+        </is>
+      </c>
+      <c r="C395" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D395" s="11" t="n">
+        <v>164</v>
+      </c>
+      <c r="E395" s="11" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="F395" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G395" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H395" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B396" s="12" t="inlineStr">
+        <is>
+          <t>14:02:41</t>
+        </is>
+      </c>
+      <c r="C396" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="D396" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E396" s="12" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="F396" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G396" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H396" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B397" s="11" t="inlineStr">
+        <is>
+          <t>14:07:45</t>
+        </is>
+      </c>
+      <c r="C397" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D397" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="E397" s="11" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="F397" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G397" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H397" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B398" s="12" t="inlineStr">
+        <is>
+          <t>14:12:48</t>
+        </is>
+      </c>
+      <c r="C398" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D398" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E398" s="12" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="F398" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G398" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="H398" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B399" s="11" t="inlineStr">
+        <is>
+          <t>14:17:52</t>
+        </is>
+      </c>
+      <c r="C399" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="D399" s="11" t="n">
+        <v>166</v>
+      </c>
+      <c r="E399" s="11" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="F399" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G399" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H399" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B400" s="12" t="inlineStr">
+        <is>
+          <t>14:22:56</t>
+        </is>
+      </c>
+      <c r="C400" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="D400" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="E400" s="12" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F400" s="12" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G400" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="H400" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B401" s="11" t="inlineStr">
+        <is>
+          <t>14:27:59</t>
+        </is>
+      </c>
+      <c r="C401" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="D401" s="11" t="n">
+        <v>165</v>
+      </c>
+      <c r="E401" s="11" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="F401" s="11" t="inlineStr">
+        <is>
+          <t>Afternoon Pickup</t>
+        </is>
+      </c>
+      <c r="G401" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H401" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B402" s="12" t="inlineStr">
+        <is>
+          <t>14:33:04</t>
+        </is>
+      </c>
+      <c r="C402" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="D402" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E402" s="12" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="F402" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G402" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H402" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B403" s="11" t="inlineStr">
+        <is>
+          <t>14:38:08</t>
+        </is>
+      </c>
+      <c r="C403" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D403" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E403" s="11" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="F403" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G403" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H403" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B404" s="12" t="inlineStr">
+        <is>
+          <t>14:43:12</t>
+        </is>
+      </c>
+      <c r="C404" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="D404" s="12" t="n">
+        <v>162</v>
+      </c>
+      <c r="E404" s="12" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="F404" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G404" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H404" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B405" s="11" t="inlineStr">
+        <is>
+          <t>14:48:16</t>
+        </is>
+      </c>
+      <c r="C405" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="D405" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E405" s="11" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="F405" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G405" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H405" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B406" s="12" t="inlineStr">
+        <is>
+          <t>14:53:19</t>
+        </is>
+      </c>
+      <c r="C406" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="D406" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="E406" s="12" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="F406" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G406" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H406" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B407" s="11" t="inlineStr">
+        <is>
+          <t>14:58:23</t>
+        </is>
+      </c>
+      <c r="C407" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="D407" s="11" t="n">
+        <v>164</v>
+      </c>
+      <c r="E407" s="11" t="n">
+        <v>51</v>
+      </c>
+      <c r="F407" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G407" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H407" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B408" s="12" t="inlineStr">
+        <is>
+          <t>15:03:28</t>
+        </is>
+      </c>
+      <c r="C408" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="D408" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="E408" s="12" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="F408" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G408" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H408" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B409" s="11" t="inlineStr">
+        <is>
+          <t>15:08:32</t>
+        </is>
+      </c>
+      <c r="C409" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D409" s="11" t="n">
+        <v>168</v>
+      </c>
+      <c r="E409" s="11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="F409" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G409" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H409" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B410" s="12" t="inlineStr">
+        <is>
+          <t>15:13:35</t>
+        </is>
+      </c>
+      <c r="C410" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="D410" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="E410" s="12" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="F410" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G410" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H410" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B411" s="11" t="inlineStr">
+        <is>
+          <t>15:18:40</t>
+        </is>
+      </c>
+      <c r="C411" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="D411" s="11" t="n">
+        <v>163</v>
+      </c>
+      <c r="E411" s="11" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="F411" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G411" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H411" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B412" s="12" t="inlineStr">
+        <is>
+          <t>15:23:44</t>
+        </is>
+      </c>
+      <c r="C412" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="D412" s="12" t="n">
+        <v>162</v>
+      </c>
+      <c r="E412" s="12" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="F412" s="12" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G412" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H412" s="12" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="11" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B413" s="11" t="inlineStr">
+        <is>
+          <t>15:28:49</t>
+        </is>
+      </c>
+      <c r="C413" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="D413" s="11" t="n">
+        <v>162</v>
+      </c>
+      <c r="E413" s="11" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="F413" s="11" t="inlineStr">
+        <is>
+          <t>Power Hour</t>
+        </is>
+      </c>
+      <c r="G413" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="H413" s="11" t="inlineStr">
+        <is>
+          <t>PAYTM, UNIONBANK, PNB, INDIANB, TMPV, KALYANKJIL, CDSL, NUVAMA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15514,7 +16542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16386,6 +17414,36 @@
         <v>0</v>
       </c>
       <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-13
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X46"/>
+  <dimension ref="A1:X47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2427,9 +2427,16 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-13  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2438,6 +2445,7 @@
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A33:X33"/>
+    <mergeCell ref="A47:X47"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A22:X22"/>
@@ -16542,7 +16550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17444,6 +17452,36 @@
         <v>0</v>
       </c>
       <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="n">
+        <v>39</v>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-14
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X47"/>
+  <dimension ref="A1:X48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2434,9 +2434,16 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-14  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2460,6 +2467,7 @@
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
+    <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A21:V21"/>
@@ -16550,7 +16558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17482,6 +17490,36 @@
         <v>0</v>
       </c>
       <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="n">
+        <v>47</v>
+      </c>
+      <c r="C31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: pre-market scan 2026-07-15 05:56 UTC
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -17536,7 +17536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18752,6 +18752,225 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>PATANJALI</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K17" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="M17" s="24" t="inlineStr"/>
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O17" s="24" t="n">
+        <v>19.92</v>
+      </c>
+      <c r="P17" s="24" t="n">
+        <v>404.9</v>
+      </c>
+      <c r="Q17" s="24" t="n">
+        <v>346.5</v>
+      </c>
+      <c r="R17" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S17" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>TATAELXSI</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="K18" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="24" t="n">
+        <v>80</v>
+      </c>
+      <c r="M18" s="24" t="inlineStr"/>
+      <c r="N18" s="24" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O18" s="24" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="P18" s="24" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="Q18" s="24" t="n">
+        <v>3461.4</v>
+      </c>
+      <c r="R18" s="24" t="inlineStr">
+        <is>
+          <t>Short Build Up</t>
+        </is>
+      </c>
+      <c r="S18" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>11:26</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>CALL</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="K19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="22" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M19" s="22" t="inlineStr"/>
+      <c r="N19" s="22" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="O19" s="22" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="P19" s="22" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="Q19" s="22" t="n">
+        <v>2020.2</v>
+      </c>
+      <c r="R19" s="22" t="inlineStr">
+        <is>
+          <t>Long Build Up</t>
+        </is>
+      </c>
+      <c r="S19" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IEP-CRED:LOW</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-15
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X48"/>
+  <dimension ref="A1:X49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2441,9 +2441,16 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-15  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="28">
+  <mergeCells count="29">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2469,6 +2476,7 @@
     <mergeCell ref="A34:X34"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A49:X49"/>
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
@@ -16558,7 +16566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17520,6 +17528,36 @@
         <v>0</v>
       </c>
       <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="n">
+        <v>46</v>
+      </c>
+      <c r="C32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-16
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X49"/>
+  <dimension ref="A1:X50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2448,14 +2448,22 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-16  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A50:X50"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A33:X33"/>
@@ -16566,7 +16574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17558,6 +17566,36 @@
         <v>0</v>
       </c>
       <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="n">
+        <v>46</v>
+      </c>
+      <c r="C33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-17
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X50"/>
+  <dimension ref="A1:X51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2455,9 +2455,16 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-17  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2485,6 +2492,7 @@
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A49:X49"/>
+    <mergeCell ref="A51:X51"/>
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
@@ -16574,7 +16582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17596,6 +17604,36 @@
         <v>0</v>
       </c>
       <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="n">
+        <v>46</v>
+      </c>
+      <c r="C34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-20
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X51"/>
+  <dimension ref="A1:X52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2462,9 +2462,16 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-20  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="31">
+  <mergeCells count="32">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2482,6 +2489,7 @@
     <mergeCell ref="A35:X35"/>
     <mergeCell ref="A43:X43"/>
     <mergeCell ref="A38:X38"/>
+    <mergeCell ref="A52:X52"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A44:X44"/>
@@ -16582,7 +16590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17634,6 +17642,36 @@
         <v>0</v>
       </c>
       <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="C35" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-21
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X52"/>
+  <dimension ref="A1:X53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2469,9 +2469,16 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-21  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="32">
+  <mergeCells count="33">
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -2485,6 +2492,7 @@
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A22:X22"/>
+    <mergeCell ref="A53:X53"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A35:X35"/>
     <mergeCell ref="A43:X43"/>
@@ -16590,7 +16598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17672,6 +17680,36 @@
         <v>0</v>
       </c>
       <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-22
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X53"/>
+  <dimension ref="A1:X54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2476,9 +2476,17 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-22  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="33">
+  <mergeCells count="34">
+    <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
@@ -16598,7 +16606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17710,6 +17718,36 @@
         <v>0</v>
       </c>
       <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-23
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X54"/>
+  <dimension ref="A1:X55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2483,15 +2483,23 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-23  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="34">
+  <mergeCells count="35">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A55:X55"/>
     <mergeCell ref="A50:X50"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A42:X42"/>
@@ -16606,7 +16614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17748,6 +17756,36 @@
         <v>0</v>
       </c>
       <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-24
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:X56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2490,14 +2490,22 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-24  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="35">
+  <mergeCells count="36">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A55:X55"/>
     <mergeCell ref="A50:X50"/>
@@ -16614,7 +16622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17786,6 +17794,36 @@
         <v>0</v>
       </c>
       <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-27
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X56"/>
+  <dimension ref="A1:X57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2497,9 +2497,16 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-27  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="36">
+  <mergeCells count="37">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2510,6 +2517,7 @@
     <mergeCell ref="A55:X55"/>
     <mergeCell ref="A50:X50"/>
     <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A57:X57"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A47:X47"/>
@@ -16622,7 +16630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17824,6 +17832,36 @@
         <v>0</v>
       </c>
       <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="n">
+        <v>37</v>
+      </c>
+      <c r="C40" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-28
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X57"/>
+  <dimension ref="A1:X58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2504,9 +2504,16 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-28  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="37">
+  <mergeCells count="38">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2533,6 +2540,7 @@
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A44:X44"/>
+    <mergeCell ref="A58:X58"/>
     <mergeCell ref="A40:X40"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
@@ -16630,7 +16638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17862,6 +17870,36 @@
         <v>0</v>
       </c>
       <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-29
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X58"/>
+  <dimension ref="A1:X59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2511,9 +2511,16 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-29  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="38">
+  <mergeCells count="39">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2545,6 +2552,7 @@
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
+    <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A49:X49"/>
@@ -16638,7 +16646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17900,6 +17908,36 @@
         <v>0</v>
       </c>
       <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-30
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X59"/>
+  <dimension ref="A1:X60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2518,9 +2518,16 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-30  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="39">
+  <mergeCells count="40">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2555,6 +2562,7 @@
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A60:X60"/>
     <mergeCell ref="A49:X49"/>
     <mergeCell ref="A51:X51"/>
     <mergeCell ref="A45:X45"/>
@@ -16646,7 +16654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17938,6 +17946,36 @@
         <v>0</v>
       </c>
       <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-07-31
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X60"/>
+  <dimension ref="A1:X61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2525,9 +2525,16 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-07-31  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="40">
+  <mergeCells count="41">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2568,6 +2575,7 @@
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
+    <mergeCell ref="A61:X61"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16654,7 +16662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17976,6 +17984,36 @@
         <v>0</v>
       </c>
       <c r="H43" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B44" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="C44" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-03
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X61"/>
+  <dimension ref="A1:X62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2532,9 +2532,16 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-03  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="41">
+  <mergeCells count="42">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2555,6 +2562,7 @@
     <mergeCell ref="A53:X53"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A35:X35"/>
+    <mergeCell ref="A62:X62"/>
     <mergeCell ref="A43:X43"/>
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A52:X52"/>
@@ -16662,7 +16670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18014,6 +18022,36 @@
         <v>0</v>
       </c>
       <c r="H44" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n">
+        <v>37</v>
+      </c>
+      <c r="C45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-04
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X62"/>
+  <dimension ref="A1:X63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2539,9 +2539,16 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-04  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="42">
+  <mergeCells count="43">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2567,6 +2574,7 @@
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A52:X52"/>
     <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A63:X63"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A44:X44"/>
     <mergeCell ref="A58:X58"/>
@@ -16670,7 +16678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18052,6 +18060,36 @@
         <v>0</v>
       </c>
       <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B46" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-05
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X63"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2546,9 +2546,16 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-05  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="43">
+  <mergeCells count="44">
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -2585,6 +2592,7 @@
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A64:X64"/>
     <mergeCell ref="A60:X60"/>
     <mergeCell ref="A49:X49"/>
     <mergeCell ref="A51:X51"/>
@@ -16678,7 +16686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18090,6 +18098,36 @@
         <v>0</v>
       </c>
       <c r="H46" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B47" s="19" t="n">
+        <v>44</v>
+      </c>
+      <c r="C47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-06
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X64"/>
+  <dimension ref="A1:X65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2553,9 +2553,17 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-06  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="44">
+  <mergeCells count="45">
+    <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -16686,7 +16694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18128,6 +18136,36 @@
         <v>0</v>
       </c>
       <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="n">
+        <v>43</v>
+      </c>
+      <c r="C48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-07
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X65"/>
+  <dimension ref="A1:X66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2560,15 +2560,23 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-07  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="45">
+  <mergeCells count="46">
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A66:X66"/>
     <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A55:X55"/>
@@ -16694,7 +16702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18166,6 +18174,36 @@
         <v>0</v>
       </c>
       <c r="H48" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="n">
+        <v>53</v>
+      </c>
+      <c r="C49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-10
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X66"/>
+  <dimension ref="A1:X67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2567,9 +2567,16 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-10  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="46">
+  <mergeCells count="47">
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
@@ -2602,6 +2609,7 @@
     <mergeCell ref="A44:X44"/>
     <mergeCell ref="A58:X58"/>
     <mergeCell ref="A40:X40"/>
+    <mergeCell ref="A67:X67"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
@@ -16702,7 +16710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18204,6 +18212,36 @@
         <v>0</v>
       </c>
       <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n">
+        <v>56</v>
+      </c>
+      <c r="C50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-11
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X67"/>
+  <dimension ref="A1:X68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2574,9 +2574,16 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-11  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="47">
+  <mergeCells count="48">
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
@@ -2604,6 +2611,7 @@
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A52:X52"/>
     <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A68:X68"/>
     <mergeCell ref="A63:X63"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A44:X44"/>
@@ -16710,7 +16718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18242,6 +18250,36 @@
         <v>0</v>
       </c>
       <c r="H50" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="n">
+        <v>60</v>
+      </c>
+      <c r="C51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-12
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X68"/>
+  <dimension ref="A1:X69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2581,9 +2581,17 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-12  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="48">
+  <mergeCells count="49">
+    <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
@@ -16718,7 +16726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18280,6 +18288,36 @@
         <v>0</v>
       </c>
       <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="C52" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-13
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X69"/>
+  <dimension ref="A1:X70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2588,9 +2588,16 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-13  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="49">
+  <mergeCells count="50">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2640,6 +2647,7 @@
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
     <mergeCell ref="A61:X61"/>
+    <mergeCell ref="A70:X70"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16726,7 +16734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18318,6 +18326,36 @@
         <v>0</v>
       </c>
       <c r="H52" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n">
+        <v>53</v>
+      </c>
+      <c r="C53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-14
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Signals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Scans" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Pre-Open" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Scans" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pre-Open" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Signals'!$A$1:$V$1</definedName>
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X70"/>
+  <dimension ref="A1:X71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2595,9 +2595,16 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-14  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="50">
+  <mergeCells count="51">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2614,6 +2621,7 @@
     <mergeCell ref="A57:X57"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A33:X33"/>
+    <mergeCell ref="A71:X71"/>
     <mergeCell ref="A47:X47"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
@@ -16734,7 +16742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18356,6 +18364,36 @@
         <v>0</v>
       </c>
       <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n">
+        <v>55</v>
+      </c>
+      <c r="C54" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-17
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X71"/>
+  <dimension ref="A1:X72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2602,9 +2602,16 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-17  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="51">
+  <mergeCells count="52">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2632,6 +2639,7 @@
     <mergeCell ref="A62:X62"/>
     <mergeCell ref="A43:X43"/>
     <mergeCell ref="A38:X38"/>
+    <mergeCell ref="A72:X72"/>
     <mergeCell ref="A52:X52"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A68:X68"/>
@@ -16742,7 +16750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18394,6 +18402,36 @@
         <v>0</v>
       </c>
       <c r="H54" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="C55" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-18
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X72"/>
+  <dimension ref="A1:X73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2609,9 +2609,16 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-18  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="52">
+  <mergeCells count="53">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2655,6 +2662,7 @@
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
+    <mergeCell ref="A73:X73"/>
     <mergeCell ref="A64:X64"/>
     <mergeCell ref="A60:X60"/>
     <mergeCell ref="A49:X49"/>
@@ -16750,7 +16758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18432,6 +18440,36 @@
         <v>0</v>
       </c>
       <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B56" s="19" t="n">
+        <v>66</v>
+      </c>
+      <c r="C56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-19
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X73"/>
+  <dimension ref="A1:X74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2616,9 +2616,16 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-19  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="53">
+  <mergeCells count="54">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2627,6 +2634,7 @@
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A66:X66"/>
+    <mergeCell ref="A74:X74"/>
     <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A55:X55"/>
@@ -16758,7 +16766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18470,6 +18478,36 @@
         <v>0</v>
       </c>
       <c r="H56" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B57" s="19" t="n">
+        <v>66</v>
+      </c>
+      <c r="C57" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-20
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X74"/>
+  <dimension ref="A1:X75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2623,9 +2623,16 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-20  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="54">
+  <mergeCells count="55">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2633,6 +2640,7 @@
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A75:X75"/>
     <mergeCell ref="A66:X66"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A56:X56"/>
@@ -16766,7 +16774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18508,6 +18516,36 @@
         <v>0</v>
       </c>
       <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="n">
+        <v>66</v>
+      </c>
+      <c r="C58" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-21
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X75"/>
+  <dimension ref="A1:X76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2630,17 +2630,24 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-21  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="55">
+  <mergeCells count="56">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
+    <mergeCell ref="A75:X75"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
-    <mergeCell ref="A75:X75"/>
     <mergeCell ref="A66:X66"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A56:X56"/>
@@ -2650,6 +2657,7 @@
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A57:X57"/>
     <mergeCell ref="A42:X42"/>
+    <mergeCell ref="A76:X76"/>
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A71:X71"/>
     <mergeCell ref="A47:X47"/>
@@ -16774,7 +16782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18546,6 +18554,36 @@
         <v>0</v>
       </c>
       <c r="H58" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B59" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="C59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-24
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X76"/>
+  <dimension ref="A1:X77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2637,9 +2637,16 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-24  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="56">
+  <mergeCells count="57">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A54:X54"/>
@@ -2683,6 +2690,7 @@
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
+    <mergeCell ref="A77:X77"/>
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
     <mergeCell ref="A24:X24"/>
@@ -16782,7 +16790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18584,6 +18592,36 @@
         <v>0</v>
       </c>
       <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B60" s="19" t="n">
+        <v>64</v>
+      </c>
+      <c r="C60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-25
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X77"/>
+  <dimension ref="A1:X78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2644,11 +2644,19 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-25  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="57">
+  <mergeCells count="58">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
+    <mergeCell ref="A78:X78"/>
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
@@ -16790,7 +16798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18622,6 +18630,36 @@
         <v>0</v>
       </c>
       <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="n">
+        <v>65</v>
+      </c>
+      <c r="C61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-08-26
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X78"/>
+  <dimension ref="A1:X79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2651,9 +2651,17 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-08-26  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="58">
+  <mergeCells count="59">
+    <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A78:X78"/>
@@ -16798,7 +16806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18660,6 +18668,36 @@
         <v>0</v>
       </c>
       <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B62" s="19" t="n">
+        <v>66</v>
+      </c>
+      <c r="C62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-01
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X79"/>
+  <dimension ref="A1:X80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2658,9 +2658,16 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-01  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="59">
+  <mergeCells count="60">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2673,6 +2680,7 @@
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A66:X66"/>
     <mergeCell ref="A74:X74"/>
+    <mergeCell ref="A80:X80"/>
     <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
     <mergeCell ref="A55:X55"/>
@@ -16806,7 +16814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18698,6 +18706,36 @@
         <v>0</v>
       </c>
       <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B63" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-02
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X80"/>
+  <dimension ref="A1:X81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2665,9 +2665,16 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-02  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="60">
+  <mergeCells count="61">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2701,6 +2708,7 @@
     <mergeCell ref="A62:X62"/>
     <mergeCell ref="A43:X43"/>
     <mergeCell ref="A38:X38"/>
+    <mergeCell ref="A81:X81"/>
     <mergeCell ref="A72:X72"/>
     <mergeCell ref="A52:X52"/>
     <mergeCell ref="A28:X28"/>
@@ -16814,7 +16822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18736,6 +18744,36 @@
         <v>0</v>
       </c>
       <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B64" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-03
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X81"/>
+  <dimension ref="A1:X82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2672,9 +2672,16 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-03  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="61">
+  <mergeCells count="62">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2728,6 +2735,7 @@
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A73:X73"/>
     <mergeCell ref="A64:X64"/>
+    <mergeCell ref="A82:X82"/>
     <mergeCell ref="A60:X60"/>
     <mergeCell ref="A49:X49"/>
     <mergeCell ref="A51:X51"/>
@@ -16822,7 +16830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18774,6 +18782,36 @@
         <v>0</v>
       </c>
       <c r="H64" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B65" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="C65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-04
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X82"/>
+  <dimension ref="A1:X83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2679,9 +2679,16 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-04  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="62">
+  <mergeCells count="63">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2732,6 +2739,7 @@
     <mergeCell ref="A77:X77"/>
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A48:X48"/>
+    <mergeCell ref="A83:X83"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A73:X73"/>
     <mergeCell ref="A64:X64"/>
@@ -16830,7 +16838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I65"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18812,6 +18820,36 @@
         <v>0</v>
       </c>
       <c r="H65" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B66" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="C66" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-07
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X83"/>
+  <dimension ref="A1:X84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2686,9 +2686,16 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-07  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="63">
+  <mergeCells count="64">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2700,6 +2707,7 @@
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A66:X66"/>
+    <mergeCell ref="A84:X84"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A80:X80"/>
     <mergeCell ref="A56:X56"/>
@@ -16838,7 +16846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18850,6 +18858,36 @@
         <v>0</v>
       </c>
       <c r="H66" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B67" s="19" t="n">
+        <v>14</v>
+      </c>
+      <c r="C67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-08
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X84"/>
+  <dimension ref="A1:X85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2693,9 +2693,16 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-08  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="64">
+  <mergeCells count="65">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2706,8 +2713,8 @@
     <mergeCell ref="A75:X75"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A84:X84"/>
     <mergeCell ref="A66:X66"/>
-    <mergeCell ref="A84:X84"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A80:X80"/>
     <mergeCell ref="A56:X56"/>
@@ -2721,6 +2728,7 @@
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A71:X71"/>
     <mergeCell ref="A47:X47"/>
+    <mergeCell ref="A85:X85"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A22:X22"/>
@@ -16846,7 +16854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18888,6 +18896,36 @@
         <v>0</v>
       </c>
       <c r="H67" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B68" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-09
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X85"/>
+  <dimension ref="A1:X86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2700,9 +2700,16 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-09  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="65">
+  <mergeCells count="66">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A65:X65"/>
@@ -2723,6 +2730,7 @@
     <mergeCell ref="A50:X50"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A57:X57"/>
+    <mergeCell ref="A86:X86"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A76:X76"/>
     <mergeCell ref="A33:X33"/>
@@ -16854,7 +16862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18926,6 +18934,36 @@
         <v>0</v>
       </c>
       <c r="H68" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B69" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-10
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X86"/>
+  <dimension ref="A1:X87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2707,11 +2707,19 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-10  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="66">
+  <mergeCells count="67">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
+    <mergeCell ref="A87:X87"/>
     <mergeCell ref="A65:X65"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A54:X54"/>
@@ -16862,7 +16870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18964,6 +18972,36 @@
         <v>0</v>
       </c>
       <c r="H69" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B70" s="19" t="n">
+        <v>17</v>
+      </c>
+      <c r="C70" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E70" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-11
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X87"/>
+  <dimension ref="A1:X88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2714,9 +2714,16 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-11  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="67">
+  <mergeCells count="68">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2783,6 +2790,7 @@
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
     <mergeCell ref="A61:X61"/>
+    <mergeCell ref="A88:X88"/>
     <mergeCell ref="A70:X70"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16870,7 +16878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:I71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19002,6 +19010,36 @@
         <v>0</v>
       </c>
       <c r="H70" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B71" s="19" t="n">
+        <v>18</v>
+      </c>
+      <c r="C71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>